<commit_message>
chore: backfill rates (22 business days)
</commit_message>
<xml_diff>
--- a/docs/data/history.xlsx
+++ b/docs/data/history.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -493,34 +493,994 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="C2" t="n">
-        <v>3.12</v>
+        <v>2.93</v>
       </c>
       <c r="D2" t="n">
-        <v>3.16</v>
+        <v>2.98</v>
       </c>
       <c r="E2" t="n">
-        <v>3.24</v>
+        <v>3.19</v>
       </c>
       <c r="F2" t="n">
-        <v>4.048</v>
+        <v>3.943</v>
       </c>
       <c r="G2" t="n">
-        <v>4.411</v>
+        <v>4.273</v>
       </c>
       <c r="H2" t="n">
-        <v>4.558</v>
+        <v>4.38</v>
       </c>
       <c r="I2" t="n">
         <v>3.66</v>
       </c>
       <c r="J2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D3" t="n">
+        <v>2.98</v>
+      </c>
+      <c r="E3" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="F3" t="n">
+        <v>3.946</v>
+      </c>
+      <c r="G3" t="n">
+        <v>4.308</v>
+      </c>
+      <c r="H3" t="n">
+        <v>4.441</v>
+      </c>
+      <c r="I3" t="n">
+        <v>3.64</v>
+      </c>
+      <c r="J3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C4" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D4" t="n">
+        <v>2.98</v>
+      </c>
+      <c r="E4" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="F4" t="n">
+        <v>3.946</v>
+      </c>
+      <c r="G4" t="n">
+        <v>4.308</v>
+      </c>
+      <c r="H4" t="n">
+        <v>4.441</v>
+      </c>
+      <c r="I4" t="n">
+        <v>3.64</v>
+      </c>
+      <c r="J4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C5" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2.98</v>
+      </c>
+      <c r="E5" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="F5" t="n">
+        <v>3.946</v>
+      </c>
+      <c r="G5" t="n">
+        <v>4.308</v>
+      </c>
+      <c r="H5" t="n">
+        <v>4.441</v>
+      </c>
+      <c r="I5" t="n">
+        <v>3.64</v>
+      </c>
+      <c r="J5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C6" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D6" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="E6" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="F6" t="n">
+        <v>3.944</v>
+      </c>
+      <c r="G6" t="n">
+        <v>4.308</v>
+      </c>
+      <c r="H6" t="n">
+        <v>4.441</v>
+      </c>
+      <c r="I6" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="J6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C7" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="E7" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="F7" t="n">
+        <v>3.958</v>
+      </c>
+      <c r="G7" t="n">
+        <v>4.324</v>
+      </c>
+      <c r="H7" t="n">
+        <v>4.465</v>
+      </c>
+      <c r="I7" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="J7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C8" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="E8" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="F8" t="n">
+        <v>3.971</v>
+      </c>
+      <c r="G8" t="n">
+        <v>4.357</v>
+      </c>
+      <c r="H8" t="n">
+        <v>4.486</v>
+      </c>
+      <c r="I8" t="n">
+        <v>3.63</v>
+      </c>
+      <c r="J8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C9" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D9" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="E9" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="F9" t="n">
+        <v>3.962</v>
+      </c>
+      <c r="G9" t="n">
+        <v>4.341</v>
+      </c>
+      <c r="H9" t="n">
+        <v>4.471</v>
+      </c>
+      <c r="I9" t="n">
+        <v>3.64</v>
+      </c>
+      <c r="J9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C10" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D10" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="E10" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="F10" t="n">
+        <v>3.961</v>
+      </c>
+      <c r="G10" t="n">
+        <v>4.348</v>
+      </c>
+      <c r="H10" t="n">
+        <v>4.464</v>
+      </c>
+      <c r="I10" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="J10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C11" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D11" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="E11" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="F11" t="n">
+        <v>3.961</v>
+      </c>
+      <c r="G11" t="n">
+        <v>4.348</v>
+      </c>
+      <c r="H11" t="n">
+        <v>4.464</v>
+      </c>
+      <c r="I11" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="J11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C12" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D12" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="E12" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="F12" t="n">
+        <v>3.961</v>
+      </c>
+      <c r="G12" t="n">
+        <v>4.348</v>
+      </c>
+      <c r="H12" t="n">
+        <v>4.464</v>
+      </c>
+      <c r="I12" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="J12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C13" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D13" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="E13" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="F13" t="n">
+        <v>3.949</v>
+      </c>
+      <c r="G13" t="n">
+        <v>4.357</v>
+      </c>
+      <c r="H13" t="n">
+        <v>4.477</v>
+      </c>
+      <c r="I13" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="J13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C14" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D14" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="E14" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="F14" t="n">
+        <v>3.949</v>
+      </c>
+      <c r="G14" t="n">
+        <v>4.357</v>
+      </c>
+      <c r="H14" t="n">
+        <v>4.477</v>
+      </c>
+      <c r="I14" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="J14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C15" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D15" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="E15" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="F15" t="n">
+        <v>3.968</v>
+      </c>
+      <c r="G15" t="n">
+        <v>4.397</v>
+      </c>
+      <c r="H15" t="n">
+        <v>4.522</v>
+      </c>
+      <c r="I15" t="n">
+        <v>3.66</v>
+      </c>
+      <c r="J15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C16" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D16" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="E16" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="F16" t="n">
+        <v>3.969</v>
+      </c>
+      <c r="G16" t="n">
+        <v>4.355</v>
+      </c>
+      <c r="H16" t="n">
+        <v>4.471</v>
+      </c>
+      <c r="I16" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="J16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C17" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D17" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="E17" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="F17" t="n">
+        <v>3.984</v>
+      </c>
+      <c r="G17" t="n">
+        <v>4.391</v>
+      </c>
+      <c r="H17" t="n">
+        <v>4.503</v>
+      </c>
+      <c r="I17" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="J17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C18" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D18" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="E18" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="F18" t="n">
+        <v>3.984</v>
+      </c>
+      <c r="G18" t="n">
+        <v>4.391</v>
+      </c>
+      <c r="H18" t="n">
+        <v>4.503</v>
+      </c>
+      <c r="I18" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="J18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C19" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D19" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="E19" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="F19" t="n">
+        <v>3.984</v>
+      </c>
+      <c r="G19" t="n">
+        <v>4.391</v>
+      </c>
+      <c r="H19" t="n">
+        <v>4.503</v>
+      </c>
+      <c r="I19" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="J19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C20" t="n">
+        <v>2.94</v>
+      </c>
+      <c r="D20" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="E20" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="F20" t="n">
+        <v>4.004</v>
+      </c>
+      <c r="G20" t="n">
+        <v>4.414</v>
+      </c>
+      <c r="H20" t="n">
+        <v>4.535</v>
+      </c>
+      <c r="I20" t="n">
+        <v>3.63</v>
+      </c>
+      <c r="J20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C21" t="n">
+        <v>2.95</v>
+      </c>
+      <c r="D21" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="E21" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="F21" t="n">
+        <v>4.006</v>
+      </c>
+      <c r="G21" t="n">
+        <v>4.396</v>
+      </c>
+      <c r="H21" t="n">
+        <v>4.516</v>
+      </c>
+      <c r="I21" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="J21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C22" t="n">
+        <v>2.95</v>
+      </c>
+      <c r="D22" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="E22" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="F22" t="n">
+        <v>4.013</v>
+      </c>
+      <c r="G22" t="n">
+        <v>4.383</v>
+      </c>
+      <c r="H22" t="n">
+        <v>4.508</v>
+      </c>
+      <c r="I22" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="J22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C23" t="n">
+        <v>2.96</v>
+      </c>
+      <c r="D23" t="n">
+        <v>3</v>
+      </c>
+      <c r="E23" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="F23" t="n">
+        <v>4.019</v>
+      </c>
+      <c r="G23" t="n">
+        <v>4.384</v>
+      </c>
+      <c r="H23" t="n">
+        <v>4.498</v>
+      </c>
+      <c r="I23" t="n">
+        <v>3.66</v>
+      </c>
+      <c r="J23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>3</v>
+      </c>
+      <c r="C24" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="D24" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="E24" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="F24" t="n">
+        <v>4.014</v>
+      </c>
+      <c r="G24" t="n">
+        <v>4.322</v>
+      </c>
+      <c r="H24" t="n">
+        <v>4.433</v>
+      </c>
+      <c r="I24" t="n">
+        <v>3.64</v>
+      </c>
+      <c r="J24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>3</v>
+      </c>
+      <c r="C25" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="D25" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="E25" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="F25" t="n">
+        <v>4.014</v>
+      </c>
+      <c r="G25" t="n">
+        <v>4.322</v>
+      </c>
+      <c r="H25" t="n">
+        <v>4.433</v>
+      </c>
+      <c r="I25" t="n">
+        <v>3.64</v>
+      </c>
+      <c r="J25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>3</v>
+      </c>
+      <c r="C26" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="D26" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="E26" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="F26" t="n">
+        <v>4.014</v>
+      </c>
+      <c r="G26" t="n">
+        <v>4.322</v>
+      </c>
+      <c r="H26" t="n">
+        <v>4.433</v>
+      </c>
+      <c r="I26" t="n">
+        <v>3.64</v>
+      </c>
+      <c r="J26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>3</v>
+      </c>
+      <c r="C27" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="D27" t="n">
+        <v>3.13</v>
+      </c>
+      <c r="E27" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="F27" t="n">
+        <v>4.019</v>
+      </c>
+      <c r="G27" t="n">
+        <v>4.368</v>
+      </c>
+      <c r="H27" t="n">
+        <v>4.476</v>
+      </c>
+      <c r="I27" t="n">
+        <v>3.64</v>
+      </c>
+      <c r="J27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>3</v>
+      </c>
+      <c r="C28" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="D28" t="n">
+        <v>3.13</v>
+      </c>
+      <c r="E28" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="F28" t="n">
+        <v>4.028</v>
+      </c>
+      <c r="G28" t="n">
+        <v>4.402</v>
+      </c>
+      <c r="H28" t="n">
+        <v>4.519</v>
+      </c>
+      <c r="I28" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="J28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>3</v>
+      </c>
+      <c r="C29" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="D29" t="n">
+        <v>3.14</v>
+      </c>
+      <c r="E29" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="F29" t="n">
+        <v>4.041</v>
+      </c>
+      <c r="G29" t="n">
+        <v>4.433</v>
+      </c>
+      <c r="H29" t="n">
+        <v>4.557</v>
+      </c>
+      <c r="I29" t="n">
+        <v>3.68</v>
+      </c>
+      <c r="J29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>3</v>
+      </c>
+      <c r="C30" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="D30" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="E30" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="F30" t="n">
+        <v>4.049</v>
+      </c>
+      <c r="G30" t="n">
+        <v>4.469</v>
+      </c>
+      <c r="H30" t="n">
+        <v>4.612</v>
+      </c>
+      <c r="I30" t="n">
+        <v>3.66</v>
+      </c>
+      <c r="J30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>3</v>
+      </c>
+      <c r="C31" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="D31" t="n">
+        <v>3.16</v>
+      </c>
+      <c r="E31" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="F31" t="n">
+        <v>4.046</v>
+      </c>
+      <c r="G31" t="n">
+        <v>4.417</v>
+      </c>
+      <c r="H31" t="n">
+        <v>4.558</v>
+      </c>
+      <c r="I31" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="J31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>3</v>
+      </c>
+      <c r="C32" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="D32" t="n">
+        <v>3.16</v>
+      </c>
+      <c r="E32" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="F32" t="n">
+        <v>4.048</v>
+      </c>
+      <c r="G32" t="n">
+        <v>4.411</v>
+      </c>
+      <c r="H32" t="n">
+        <v>4.558</v>
+      </c>
+      <c r="I32" t="n">
+        <v>3.66</v>
+      </c>
+      <c r="J32" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: update rates (2026-09-07 17:01 KST)
</commit_message>
<xml_diff>
--- a/docs/data/history.xlsx
+++ b/docs/data/history.xlsx
@@ -1537,7 +1537,9 @@
       <c r="H32" t="n">
         <v>4.558</v>
       </c>
-      <c r="I32" t="inlineStr"/>
+      <c r="I32" t="n">
+        <v>3.885</v>
+      </c>
       <c r="J32" t="n">
         <v>3.66</v>
       </c>
@@ -1569,7 +1571,9 @@
       <c r="H33" t="n">
         <v>4.558</v>
       </c>
-      <c r="I33" t="inlineStr"/>
+      <c r="I33" t="n">
+        <v>3.885</v>
+      </c>
       <c r="J33" t="n">
         <v>3.66</v>
       </c>
@@ -1601,7 +1605,9 @@
       <c r="H34" t="n">
         <v>4.558</v>
       </c>
-      <c r="I34" t="inlineStr"/>
+      <c r="I34" t="n">
+        <v>3.885</v>
+      </c>
       <c r="J34" t="n">
         <v>3.66</v>
       </c>

</xml_diff>

<commit_message>
chore: update rates (2026-09-08 08:12 KST)
</commit_message>
<xml_diff>
--- a/docs/data/history.xlsx
+++ b/docs/data/history.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J34"/>
+  <dimension ref="A1:J35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -493,7 +493,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -527,7 +527,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -561,7 +561,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -595,7 +595,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -629,7 +629,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -663,7 +663,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -697,7 +697,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -731,7 +731,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -765,7 +765,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -799,7 +799,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -833,7 +833,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -867,7 +867,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -901,7 +901,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -935,7 +935,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -969,7 +969,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -1003,7 +1003,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1037,7 +1037,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -1071,7 +1071,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1105,7 +1105,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -1139,7 +1139,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1173,7 +1173,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -1207,7 +1207,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1241,7 +1241,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1275,7 +1275,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1309,7 +1309,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1343,7 +1343,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1377,7 +1377,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1411,7 +1411,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1445,7 +1445,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1479,7 +1479,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1513,7 +1513,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1547,7 +1547,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1581,7 +1581,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1609,6 +1609,40 @@
         <v>3.885</v>
       </c>
       <c r="J34" t="n">
+        <v>3.66</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>3</v>
+      </c>
+      <c r="C35" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="D35" t="n">
+        <v>3.16</v>
+      </c>
+      <c r="E35" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="F35" t="n">
+        <v>4.054</v>
+      </c>
+      <c r="G35" t="n">
+        <v>4.43</v>
+      </c>
+      <c r="H35" t="n">
+        <v>4.57</v>
+      </c>
+      <c r="I35" t="n">
+        <v>3.897</v>
+      </c>
+      <c r="J35" t="n">
         <v>3.66</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update rates (2026-09-09 08:19 KST)
</commit_message>
<xml_diff>
--- a/docs/data/history.xlsx
+++ b/docs/data/history.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J35"/>
+  <dimension ref="A1:J36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -456,12 +456,12 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>A1CP(3개월)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>A1CP(1개월)</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>A1CP(3개월)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -503,10 +503,10 @@
         <v>2.93</v>
       </c>
       <c r="D2" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E2" t="n">
         <v>2.98</v>
-      </c>
-      <c r="E2" t="n">
-        <v>3.19</v>
       </c>
       <c r="F2" t="n">
         <v>3.943</v>
@@ -537,10 +537,10 @@
         <v>2.93</v>
       </c>
       <c r="D3" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E3" t="n">
         <v>2.98</v>
-      </c>
-      <c r="E3" t="n">
-        <v>3.19</v>
       </c>
       <c r="F3" t="n">
         <v>3.946</v>
@@ -571,10 +571,10 @@
         <v>2.93</v>
       </c>
       <c r="D4" t="n">
-        <v>2.99</v>
+        <v>3.19</v>
       </c>
       <c r="E4" t="n">
-        <v>3.19</v>
+        <v>2.99</v>
       </c>
       <c r="F4" t="n">
         <v>3.944</v>
@@ -605,10 +605,10 @@
         <v>2.93</v>
       </c>
       <c r="D5" t="n">
-        <v>2.99</v>
+        <v>3.19</v>
       </c>
       <c r="E5" t="n">
-        <v>3.19</v>
+        <v>2.99</v>
       </c>
       <c r="F5" t="n">
         <v>3.944</v>
@@ -639,10 +639,10 @@
         <v>2.93</v>
       </c>
       <c r="D6" t="n">
-        <v>2.99</v>
+        <v>3.19</v>
       </c>
       <c r="E6" t="n">
-        <v>3.19</v>
+        <v>2.99</v>
       </c>
       <c r="F6" t="n">
         <v>3.944</v>
@@ -673,10 +673,10 @@
         <v>2.93</v>
       </c>
       <c r="D7" t="n">
-        <v>2.99</v>
+        <v>3.19</v>
       </c>
       <c r="E7" t="n">
-        <v>3.19</v>
+        <v>2.99</v>
       </c>
       <c r="F7" t="n">
         <v>3.958</v>
@@ -707,10 +707,10 @@
         <v>2.93</v>
       </c>
       <c r="D8" t="n">
-        <v>2.99</v>
+        <v>3.19</v>
       </c>
       <c r="E8" t="n">
-        <v>3.19</v>
+        <v>2.99</v>
       </c>
       <c r="F8" t="n">
         <v>3.971</v>
@@ -741,10 +741,10 @@
         <v>2.93</v>
       </c>
       <c r="D9" t="n">
-        <v>2.99</v>
+        <v>3.19</v>
       </c>
       <c r="E9" t="n">
-        <v>3.19</v>
+        <v>2.99</v>
       </c>
       <c r="F9" t="n">
         <v>3.962</v>
@@ -775,10 +775,10 @@
         <v>2.93</v>
       </c>
       <c r="D10" t="n">
-        <v>2.99</v>
+        <v>3.19</v>
       </c>
       <c r="E10" t="n">
-        <v>3.19</v>
+        <v>2.99</v>
       </c>
       <c r="F10" t="n">
         <v>3.961</v>
@@ -809,10 +809,10 @@
         <v>2.93</v>
       </c>
       <c r="D11" t="n">
-        <v>2.99</v>
+        <v>3.19</v>
       </c>
       <c r="E11" t="n">
-        <v>3.19</v>
+        <v>2.99</v>
       </c>
       <c r="F11" t="n">
         <v>3.949</v>
@@ -843,10 +843,10 @@
         <v>2.93</v>
       </c>
       <c r="D12" t="n">
-        <v>2.99</v>
+        <v>3.19</v>
       </c>
       <c r="E12" t="n">
-        <v>3.19</v>
+        <v>2.99</v>
       </c>
       <c r="F12" t="n">
         <v>3.949</v>
@@ -877,10 +877,10 @@
         <v>2.93</v>
       </c>
       <c r="D13" t="n">
-        <v>2.99</v>
+        <v>3.19</v>
       </c>
       <c r="E13" t="n">
-        <v>3.19</v>
+        <v>2.99</v>
       </c>
       <c r="F13" t="n">
         <v>3.949</v>
@@ -911,10 +911,10 @@
         <v>2.93</v>
       </c>
       <c r="D14" t="n">
-        <v>2.99</v>
+        <v>3.19</v>
       </c>
       <c r="E14" t="n">
-        <v>3.19</v>
+        <v>2.99</v>
       </c>
       <c r="F14" t="n">
         <v>3.949</v>
@@ -945,10 +945,10 @@
         <v>2.93</v>
       </c>
       <c r="D15" t="n">
-        <v>2.99</v>
+        <v>3.19</v>
       </c>
       <c r="E15" t="n">
-        <v>3.19</v>
+        <v>2.99</v>
       </c>
       <c r="F15" t="n">
         <v>3.968</v>
@@ -979,10 +979,10 @@
         <v>2.93</v>
       </c>
       <c r="D16" t="n">
-        <v>2.99</v>
+        <v>3.19</v>
       </c>
       <c r="E16" t="n">
-        <v>3.19</v>
+        <v>2.99</v>
       </c>
       <c r="F16" t="n">
         <v>3.969</v>
@@ -1013,10 +1013,10 @@
         <v>2.93</v>
       </c>
       <c r="D17" t="n">
-        <v>2.99</v>
+        <v>3.19</v>
       </c>
       <c r="E17" t="n">
-        <v>3.19</v>
+        <v>2.99</v>
       </c>
       <c r="F17" t="n">
         <v>3.984</v>
@@ -1047,10 +1047,10 @@
         <v>2.94</v>
       </c>
       <c r="D18" t="n">
-        <v>2.99</v>
+        <v>3.19</v>
       </c>
       <c r="E18" t="n">
-        <v>3.19</v>
+        <v>2.99</v>
       </c>
       <c r="F18" t="n">
         <v>4.004</v>
@@ -1081,10 +1081,10 @@
         <v>2.94</v>
       </c>
       <c r="D19" t="n">
-        <v>2.99</v>
+        <v>3.19</v>
       </c>
       <c r="E19" t="n">
-        <v>3.19</v>
+        <v>2.99</v>
       </c>
       <c r="F19" t="n">
         <v>4.004</v>
@@ -1115,10 +1115,10 @@
         <v>2.94</v>
       </c>
       <c r="D20" t="n">
-        <v>2.99</v>
+        <v>3.19</v>
       </c>
       <c r="E20" t="n">
-        <v>3.19</v>
+        <v>2.99</v>
       </c>
       <c r="F20" t="n">
         <v>4.004</v>
@@ -1149,10 +1149,10 @@
         <v>2.95</v>
       </c>
       <c r="D21" t="n">
-        <v>2.99</v>
+        <v>3.19</v>
       </c>
       <c r="E21" t="n">
-        <v>3.19</v>
+        <v>2.99</v>
       </c>
       <c r="F21" t="n">
         <v>4.006</v>
@@ -1183,10 +1183,10 @@
         <v>2.95</v>
       </c>
       <c r="D22" t="n">
-        <v>2.99</v>
+        <v>3.19</v>
       </c>
       <c r="E22" t="n">
-        <v>3.19</v>
+        <v>2.99</v>
       </c>
       <c r="F22" t="n">
         <v>4.013</v>
@@ -1217,10 +1217,10 @@
         <v>2.96</v>
       </c>
       <c r="D23" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="E23" t="n">
         <v>3</v>
-      </c>
-      <c r="E23" t="n">
-        <v>3.2</v>
       </c>
       <c r="F23" t="n">
         <v>4.019</v>
@@ -1251,10 +1251,10 @@
         <v>3.12</v>
       </c>
       <c r="D24" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="E24" t="n">
         <v>3.12</v>
-      </c>
-      <c r="E24" t="n">
-        <v>3.23</v>
       </c>
       <c r="F24" t="n">
         <v>4.014</v>
@@ -1285,10 +1285,10 @@
         <v>3.12</v>
       </c>
       <c r="D25" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="E25" t="n">
         <v>3.13</v>
-      </c>
-      <c r="E25" t="n">
-        <v>3.23</v>
       </c>
       <c r="F25" t="n">
         <v>4.019</v>
@@ -1319,10 +1319,10 @@
         <v>3.12</v>
       </c>
       <c r="D26" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="E26" t="n">
         <v>3.13</v>
-      </c>
-      <c r="E26" t="n">
-        <v>3.23</v>
       </c>
       <c r="F26" t="n">
         <v>4.019</v>
@@ -1353,10 +1353,10 @@
         <v>3.12</v>
       </c>
       <c r="D27" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="E27" t="n">
         <v>3.13</v>
-      </c>
-      <c r="E27" t="n">
-        <v>3.23</v>
       </c>
       <c r="F27" t="n">
         <v>4.019</v>
@@ -1387,10 +1387,10 @@
         <v>3.12</v>
       </c>
       <c r="D28" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="E28" t="n">
         <v>3.13</v>
-      </c>
-      <c r="E28" t="n">
-        <v>3.23</v>
       </c>
       <c r="F28" t="n">
         <v>4.028</v>
@@ -1421,10 +1421,10 @@
         <v>3.12</v>
       </c>
       <c r="D29" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="E29" t="n">
         <v>3.14</v>
-      </c>
-      <c r="E29" t="n">
-        <v>3.23</v>
       </c>
       <c r="F29" t="n">
         <v>4.041</v>
@@ -1455,10 +1455,10 @@
         <v>3.12</v>
       </c>
       <c r="D30" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="E30" t="n">
         <v>3.15</v>
-      </c>
-      <c r="E30" t="n">
-        <v>3.23</v>
       </c>
       <c r="F30" t="n">
         <v>4.049</v>
@@ -1489,10 +1489,10 @@
         <v>3.12</v>
       </c>
       <c r="D31" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="E31" t="n">
         <v>3.16</v>
-      </c>
-      <c r="E31" t="n">
-        <v>3.24</v>
       </c>
       <c r="F31" t="n">
         <v>4.046</v>
@@ -1523,10 +1523,10 @@
         <v>3.12</v>
       </c>
       <c r="D32" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="E32" t="n">
         <v>3.16</v>
-      </c>
-      <c r="E32" t="n">
-        <v>3.24</v>
       </c>
       <c r="F32" t="n">
         <v>4.048</v>
@@ -1557,10 +1557,10 @@
         <v>3.12</v>
       </c>
       <c r="D33" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="E33" t="n">
         <v>3.16</v>
-      </c>
-      <c r="E33" t="n">
-        <v>3.24</v>
       </c>
       <c r="F33" t="n">
         <v>4.048</v>
@@ -1591,10 +1591,10 @@
         <v>3.12</v>
       </c>
       <c r="D34" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="E34" t="n">
         <v>3.16</v>
-      </c>
-      <c r="E34" t="n">
-        <v>3.24</v>
       </c>
       <c r="F34" t="n">
         <v>4.048</v>
@@ -1625,10 +1625,10 @@
         <v>3.12</v>
       </c>
       <c r="D35" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="E35" t="n">
         <v>3.16</v>
-      </c>
-      <c r="E35" t="n">
-        <v>3.24</v>
       </c>
       <c r="F35" t="n">
         <v>4.054</v>
@@ -1644,6 +1644,40 @@
       </c>
       <c r="J35" t="n">
         <v>3.66</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>3</v>
+      </c>
+      <c r="C36" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="D36" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="E36" t="n">
+        <v>3.17</v>
+      </c>
+      <c r="F36" t="n">
+        <v>4.069</v>
+      </c>
+      <c r="G36" t="n">
+        <v>4.438</v>
+      </c>
+      <c r="H36" t="n">
+        <v>4.568</v>
+      </c>
+      <c r="I36" t="n">
+        <v>3.897</v>
+      </c>
+      <c r="J36" t="n">
+        <v>3.65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update rates (2026-09-10 07:55 KST)
</commit_message>
<xml_diff>
--- a/docs/data/history.xlsx
+++ b/docs/data/history.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J36"/>
+  <dimension ref="A1:J37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1680,6 +1680,40 @@
         <v>3.65</v>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>3</v>
+      </c>
+      <c r="C37" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="D37" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="E37" t="n">
+        <v>3.18</v>
+      </c>
+      <c r="F37" t="n">
+        <v>4.078</v>
+      </c>
+      <c r="G37" t="n">
+        <v>4.445</v>
+      </c>
+      <c r="H37" t="n">
+        <v>4.58</v>
+      </c>
+      <c r="I37" t="n">
+        <v>3.91</v>
+      </c>
+      <c r="J37" t="n">
+        <v>3.64</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update rates (2026-09-11 07:56 KST)
</commit_message>
<xml_diff>
--- a/docs/data/history.xlsx
+++ b/docs/data/history.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J37"/>
+  <dimension ref="A1:J38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1714,6 +1714,40 @@
         <v>3.64</v>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>3</v>
+      </c>
+      <c r="C38" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="D38" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="E38" t="n">
+        <v>3.18</v>
+      </c>
+      <c r="F38" t="n">
+        <v>4.091</v>
+      </c>
+      <c r="G38" t="n">
+        <v>4.464</v>
+      </c>
+      <c r="H38" t="n">
+        <v>4.595</v>
+      </c>
+      <c r="I38" t="n">
+        <v>3.927</v>
+      </c>
+      <c r="J38" t="n">
+        <v>3.64</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: backfill rates (50 business days)
</commit_message>
<xml_diff>
--- a/docs/data/history.xlsx
+++ b/docs/data/history.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J38"/>
+  <dimension ref="A1:J71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -493,63 +493,63 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C2" t="n">
-        <v>2.93</v>
+        <v>2.92</v>
       </c>
       <c r="D2" t="n">
         <v>3.19</v>
       </c>
       <c r="E2" t="n">
-        <v>2.98</v>
+        <v>2.96</v>
       </c>
       <c r="F2" t="n">
-        <v>3.943</v>
+        <v>3.973</v>
       </c>
       <c r="G2" t="n">
-        <v>4.273</v>
+        <v>4.4</v>
       </c>
       <c r="H2" t="n">
-        <v>4.38</v>
+        <v>4.437</v>
       </c>
       <c r="I2" t="n">
-        <v>3.677</v>
+        <v>3.745</v>
       </c>
       <c r="J2" t="n">
-        <v>3.66</v>
+        <v>3.64</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C3" t="n">
-        <v>2.93</v>
+        <v>2.92</v>
       </c>
       <c r="D3" t="n">
         <v>3.19</v>
       </c>
       <c r="E3" t="n">
-        <v>2.98</v>
+        <v>2.96</v>
       </c>
       <c r="F3" t="n">
-        <v>3.946</v>
+        <v>3.973</v>
       </c>
       <c r="G3" t="n">
-        <v>4.308</v>
+        <v>4.4</v>
       </c>
       <c r="H3" t="n">
-        <v>4.441</v>
+        <v>4.437</v>
       </c>
       <c r="I3" t="n">
         <v>3.745</v>
@@ -561,134 +561,134 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C4" t="n">
-        <v>2.93</v>
+        <v>2.92</v>
       </c>
       <c r="D4" t="n">
         <v>3.19</v>
       </c>
       <c r="E4" t="n">
-        <v>2.99</v>
+        <v>2.96</v>
       </c>
       <c r="F4" t="n">
-        <v>3.944</v>
+        <v>3.973</v>
       </c>
       <c r="G4" t="n">
-        <v>4.308</v>
+        <v>4.4</v>
       </c>
       <c r="H4" t="n">
-        <v>4.441</v>
+        <v>4.437</v>
       </c>
       <c r="I4" t="n">
-        <v>3.747</v>
+        <v>3.745</v>
       </c>
       <c r="J4" t="n">
-        <v>3.65</v>
+        <v>3.64</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C5" t="n">
-        <v>2.93</v>
+        <v>2.92</v>
       </c>
       <c r="D5" t="n">
         <v>3.19</v>
       </c>
       <c r="E5" t="n">
-        <v>2.99</v>
+        <v>2.95</v>
       </c>
       <c r="F5" t="n">
-        <v>3.944</v>
+        <v>3.976</v>
       </c>
       <c r="G5" t="n">
-        <v>4.308</v>
+        <v>4.401</v>
       </c>
       <c r="H5" t="n">
-        <v>4.441</v>
+        <v>4.461</v>
       </c>
       <c r="I5" t="n">
-        <v>3.747</v>
+        <v>3.77</v>
       </c>
       <c r="J5" t="n">
-        <v>3.65</v>
+        <v>3.64</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C6" t="n">
-        <v>2.93</v>
+        <v>2.91</v>
       </c>
       <c r="D6" t="n">
-        <v>3.19</v>
+        <v>3.18</v>
       </c>
       <c r="E6" t="n">
-        <v>2.99</v>
+        <v>2.94</v>
       </c>
       <c r="F6" t="n">
-        <v>3.944</v>
+        <v>3.977</v>
       </c>
       <c r="G6" t="n">
-        <v>4.308</v>
+        <v>4.399</v>
       </c>
       <c r="H6" t="n">
-        <v>4.441</v>
+        <v>4.469</v>
       </c>
       <c r="I6" t="n">
-        <v>3.747</v>
+        <v>3.777</v>
       </c>
       <c r="J6" t="n">
-        <v>3.65</v>
+        <v>3.63</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C7" t="n">
-        <v>2.93</v>
+        <v>2.91</v>
       </c>
       <c r="D7" t="n">
-        <v>3.19</v>
+        <v>3.18</v>
       </c>
       <c r="E7" t="n">
-        <v>2.99</v>
+        <v>2.94</v>
       </c>
       <c r="F7" t="n">
-        <v>3.958</v>
+        <v>3.986</v>
       </c>
       <c r="G7" t="n">
-        <v>4.324</v>
+        <v>4.395</v>
       </c>
       <c r="H7" t="n">
-        <v>4.465</v>
+        <v>4.472</v>
       </c>
       <c r="I7" t="n">
-        <v>3.775</v>
+        <v>3.776</v>
       </c>
       <c r="J7" t="n">
         <v>3.62</v>
@@ -697,338 +697,338 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C8" t="n">
+        <v>2.91</v>
+      </c>
+      <c r="D8" t="n">
+        <v>3.18</v>
+      </c>
+      <c r="E8" t="n">
         <v>2.93</v>
       </c>
-      <c r="D8" t="n">
-        <v>3.19</v>
-      </c>
-      <c r="E8" t="n">
-        <v>2.99</v>
-      </c>
       <c r="F8" t="n">
-        <v>3.971</v>
+        <v>3.991</v>
       </c>
       <c r="G8" t="n">
-        <v>4.357</v>
+        <v>4.407</v>
       </c>
       <c r="H8" t="n">
-        <v>4.486</v>
+        <v>4.478</v>
       </c>
       <c r="I8" t="n">
-        <v>3.797</v>
+        <v>3.78</v>
       </c>
       <c r="J8" t="n">
-        <v>3.63</v>
+        <v>3.58</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C9" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="D9" t="n">
+        <v>3.17</v>
+      </c>
+      <c r="E9" t="n">
         <v>2.93</v>
       </c>
-      <c r="D9" t="n">
-        <v>3.19</v>
-      </c>
-      <c r="E9" t="n">
-        <v>2.99</v>
-      </c>
       <c r="F9" t="n">
-        <v>3.962</v>
+        <v>3.997</v>
       </c>
       <c r="G9" t="n">
-        <v>4.341</v>
+        <v>4.399</v>
       </c>
       <c r="H9" t="n">
-        <v>4.471</v>
+        <v>4.47</v>
       </c>
       <c r="I9" t="n">
-        <v>3.782</v>
+        <v>3.77</v>
       </c>
       <c r="J9" t="n">
-        <v>3.64</v>
+        <v>3.53</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C10" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="D10" t="n">
+        <v>3.17</v>
+      </c>
+      <c r="E10" t="n">
         <v>2.93</v>
       </c>
-      <c r="D10" t="n">
-        <v>3.19</v>
-      </c>
-      <c r="E10" t="n">
-        <v>2.99</v>
-      </c>
       <c r="F10" t="n">
-        <v>3.961</v>
+        <v>3.997</v>
       </c>
       <c r="G10" t="n">
-        <v>4.348</v>
+        <v>4.399</v>
       </c>
       <c r="H10" t="n">
-        <v>4.464</v>
+        <v>4.47</v>
       </c>
       <c r="I10" t="n">
-        <v>3.777</v>
+        <v>3.77</v>
       </c>
       <c r="J10" t="n">
-        <v>3.62</v>
+        <v>3.53</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C11" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="D11" t="n">
+        <v>3.17</v>
+      </c>
+      <c r="E11" t="n">
         <v>2.93</v>
       </c>
-      <c r="D11" t="n">
-        <v>3.19</v>
-      </c>
-      <c r="E11" t="n">
-        <v>2.99</v>
-      </c>
       <c r="F11" t="n">
-        <v>3.949</v>
+        <v>3.997</v>
       </c>
       <c r="G11" t="n">
-        <v>4.357</v>
+        <v>4.399</v>
       </c>
       <c r="H11" t="n">
-        <v>4.477</v>
+        <v>4.47</v>
       </c>
       <c r="I11" t="n">
-        <v>3.795</v>
+        <v>3.77</v>
       </c>
       <c r="J11" t="n">
-        <v>3.62</v>
+        <v>3.53</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C12" t="n">
-        <v>2.93</v>
+        <v>2.9</v>
       </c>
       <c r="D12" t="n">
-        <v>3.19</v>
+        <v>3.17</v>
       </c>
       <c r="E12" t="n">
-        <v>2.99</v>
+        <v>2.92</v>
       </c>
       <c r="F12" t="n">
-        <v>3.949</v>
+        <v>4.009</v>
       </c>
       <c r="G12" t="n">
-        <v>4.357</v>
+        <v>4.429</v>
       </c>
       <c r="H12" t="n">
-        <v>4.477</v>
+        <v>4.513</v>
       </c>
       <c r="I12" t="n">
-        <v>3.795</v>
+        <v>3.81</v>
       </c>
       <c r="J12" t="n">
-        <v>3.62</v>
+        <v>3.55</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C13" t="n">
-        <v>2.93</v>
+        <v>2.9</v>
       </c>
       <c r="D13" t="n">
-        <v>3.19</v>
+        <v>3.17</v>
       </c>
       <c r="E13" t="n">
-        <v>2.99</v>
+        <v>2.92</v>
       </c>
       <c r="F13" t="n">
-        <v>3.949</v>
+        <v>4.036</v>
       </c>
       <c r="G13" t="n">
-        <v>4.357</v>
+        <v>4.489</v>
       </c>
       <c r="H13" t="n">
-        <v>4.477</v>
+        <v>4.594</v>
       </c>
       <c r="I13" t="n">
-        <v>3.795</v>
+        <v>3.89</v>
       </c>
       <c r="J13" t="n">
-        <v>3.62</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C14" t="n">
-        <v>2.93</v>
+        <v>2.9</v>
       </c>
       <c r="D14" t="n">
-        <v>3.19</v>
+        <v>3.17</v>
       </c>
       <c r="E14" t="n">
-        <v>2.99</v>
+        <v>2.92</v>
       </c>
       <c r="F14" t="n">
-        <v>3.949</v>
+        <v>4.018</v>
       </c>
       <c r="G14" t="n">
-        <v>4.357</v>
+        <v>4.462</v>
       </c>
       <c r="H14" t="n">
-        <v>4.477</v>
+        <v>4.572</v>
       </c>
       <c r="I14" t="n">
-        <v>3.795</v>
+        <v>3.867</v>
       </c>
       <c r="J14" t="n">
-        <v>3.62</v>
+        <v>3.63</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B15" t="n">
         <v>2.75</v>
       </c>
       <c r="C15" t="n">
-        <v>2.93</v>
+        <v>2.9</v>
       </c>
       <c r="D15" t="n">
-        <v>3.19</v>
+        <v>3.17</v>
       </c>
       <c r="E15" t="n">
-        <v>2.99</v>
+        <v>2.97</v>
       </c>
       <c r="F15" t="n">
-        <v>3.968</v>
+        <v>3.992</v>
       </c>
       <c r="G15" t="n">
-        <v>4.397</v>
+        <v>4.424</v>
       </c>
       <c r="H15" t="n">
-        <v>4.522</v>
+        <v>4.554</v>
       </c>
       <c r="I15" t="n">
-        <v>3.84</v>
+        <v>3.852</v>
       </c>
       <c r="J15" t="n">
-        <v>3.66</v>
+        <v>3.64</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B16" t="n">
         <v>2.75</v>
       </c>
       <c r="C16" t="n">
-        <v>2.93</v>
+        <v>2.9</v>
       </c>
       <c r="D16" t="n">
-        <v>3.19</v>
+        <v>3.17</v>
       </c>
       <c r="E16" t="n">
-        <v>2.99</v>
+        <v>2.97</v>
       </c>
       <c r="F16" t="n">
-        <v>3.969</v>
+        <v>3.992</v>
       </c>
       <c r="G16" t="n">
-        <v>4.355</v>
+        <v>4.424</v>
       </c>
       <c r="H16" t="n">
-        <v>4.471</v>
+        <v>4.554</v>
       </c>
       <c r="I16" t="n">
-        <v>3.787</v>
+        <v>3.852</v>
       </c>
       <c r="J16" t="n">
-        <v>3.65</v>
+        <v>3.62</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B17" t="n">
         <v>2.75</v>
       </c>
       <c r="C17" t="n">
-        <v>2.93</v>
+        <v>2.9</v>
       </c>
       <c r="D17" t="n">
-        <v>3.19</v>
+        <v>3.17</v>
       </c>
       <c r="E17" t="n">
-        <v>2.99</v>
+        <v>2.97</v>
       </c>
       <c r="F17" t="n">
-        <v>3.984</v>
+        <v>3.992</v>
       </c>
       <c r="G17" t="n">
-        <v>4.391</v>
+        <v>4.424</v>
       </c>
       <c r="H17" t="n">
-        <v>4.503</v>
+        <v>4.554</v>
       </c>
       <c r="I17" t="n">
-        <v>3.822</v>
+        <v>3.852</v>
       </c>
       <c r="J17" t="n">
         <v>3.62</v>
@@ -1037,236 +1037,236 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B18" t="n">
         <v>2.75</v>
       </c>
       <c r="C18" t="n">
-        <v>2.94</v>
+        <v>2.9</v>
       </c>
       <c r="D18" t="n">
-        <v>3.19</v>
+        <v>3.17</v>
       </c>
       <c r="E18" t="n">
-        <v>2.99</v>
+        <v>2.97</v>
       </c>
       <c r="F18" t="n">
-        <v>4.004</v>
+        <v>3.992</v>
       </c>
       <c r="G18" t="n">
-        <v>4.414</v>
+        <v>4.424</v>
       </c>
       <c r="H18" t="n">
-        <v>4.535</v>
+        <v>4.554</v>
       </c>
       <c r="I18" t="n">
-        <v>3.855</v>
+        <v>3.852</v>
       </c>
       <c r="J18" t="n">
-        <v>3.63</v>
+        <v>3.62</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B19" t="n">
         <v>2.75</v>
       </c>
       <c r="C19" t="n">
-        <v>2.94</v>
+        <v>2.91</v>
       </c>
       <c r="D19" t="n">
-        <v>3.19</v>
+        <v>3.18</v>
       </c>
       <c r="E19" t="n">
-        <v>2.99</v>
+        <v>2.98</v>
       </c>
       <c r="F19" t="n">
-        <v>4.004</v>
+        <v>4.003</v>
       </c>
       <c r="G19" t="n">
-        <v>4.414</v>
+        <v>4.452</v>
       </c>
       <c r="H19" t="n">
-        <v>4.535</v>
+        <v>4.599</v>
       </c>
       <c r="I19" t="n">
-        <v>3.855</v>
+        <v>3.897</v>
       </c>
       <c r="J19" t="n">
-        <v>3.63</v>
+        <v>3.59</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B20" t="n">
         <v>2.75</v>
       </c>
       <c r="C20" t="n">
-        <v>2.94</v>
+        <v>2.91</v>
       </c>
       <c r="D20" t="n">
         <v>3.19</v>
       </c>
       <c r="E20" t="n">
-        <v>2.99</v>
+        <v>2.98</v>
       </c>
       <c r="F20" t="n">
-        <v>4.004</v>
+        <v>3.988</v>
       </c>
       <c r="G20" t="n">
-        <v>4.414</v>
+        <v>4.398</v>
       </c>
       <c r="H20" t="n">
-        <v>4.535</v>
+        <v>4.57</v>
       </c>
       <c r="I20" t="n">
-        <v>3.855</v>
+        <v>3.866</v>
       </c>
       <c r="J20" t="n">
-        <v>3.63</v>
+        <v>3.57</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>2.75</v>
       </c>
       <c r="C21" t="n">
-        <v>2.95</v>
+        <v>2.91</v>
       </c>
       <c r="D21" t="n">
         <v>3.19</v>
       </c>
       <c r="E21" t="n">
-        <v>2.99</v>
+        <v>2.98</v>
       </c>
       <c r="F21" t="n">
-        <v>4.006</v>
+        <v>3.999</v>
       </c>
       <c r="G21" t="n">
-        <v>4.396</v>
+        <v>4.444</v>
       </c>
       <c r="H21" t="n">
-        <v>4.516</v>
+        <v>4.617</v>
       </c>
       <c r="I21" t="n">
-        <v>3.835</v>
+        <v>3.915</v>
       </c>
       <c r="J21" t="n">
-        <v>3.65</v>
+        <v>3.61</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B22" t="n">
         <v>2.75</v>
       </c>
       <c r="C22" t="n">
-        <v>2.95</v>
+        <v>2.91</v>
       </c>
       <c r="D22" t="n">
         <v>3.19</v>
       </c>
       <c r="E22" t="n">
-        <v>2.99</v>
+        <v>2.98</v>
       </c>
       <c r="F22" t="n">
-        <v>4.013</v>
+        <v>4.007</v>
       </c>
       <c r="G22" t="n">
-        <v>4.383</v>
+        <v>4.454</v>
       </c>
       <c r="H22" t="n">
-        <v>4.508</v>
+        <v>4.617</v>
       </c>
       <c r="I22" t="n">
-        <v>3.826</v>
+        <v>3.917</v>
       </c>
       <c r="J22" t="n">
-        <v>3.65</v>
+        <v>3.62</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B23" t="n">
         <v>2.75</v>
       </c>
       <c r="C23" t="n">
-        <v>2.96</v>
+        <v>2.91</v>
       </c>
       <c r="D23" t="n">
-        <v>3.2</v>
+        <v>3.19</v>
       </c>
       <c r="E23" t="n">
-        <v>3</v>
+        <v>2.98</v>
       </c>
       <c r="F23" t="n">
-        <v>4.019</v>
+        <v>4.017</v>
       </c>
       <c r="G23" t="n">
-        <v>4.384</v>
+        <v>4.482</v>
       </c>
       <c r="H23" t="n">
-        <v>4.498</v>
+        <v>4.653</v>
       </c>
       <c r="I23" t="n">
-        <v>3.817</v>
+        <v>3.952</v>
       </c>
       <c r="J23" t="n">
-        <v>3.66</v>
+        <v>3.64</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="C24" t="n">
-        <v>3.12</v>
+        <v>2.91</v>
       </c>
       <c r="D24" t="n">
-        <v>3.23</v>
+        <v>3.19</v>
       </c>
       <c r="E24" t="n">
-        <v>3.12</v>
+        <v>2.98</v>
       </c>
       <c r="F24" t="n">
-        <v>4.014</v>
+        <v>4.017</v>
       </c>
       <c r="G24" t="n">
-        <v>4.322</v>
+        <v>4.482</v>
       </c>
       <c r="H24" t="n">
-        <v>4.433</v>
+        <v>4.653</v>
       </c>
       <c r="I24" t="n">
-        <v>3.75</v>
+        <v>3.952</v>
       </c>
       <c r="J24" t="n">
         <v>3.64</v>
@@ -1275,32 +1275,32 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="C25" t="n">
-        <v>3.12</v>
+        <v>2.91</v>
       </c>
       <c r="D25" t="n">
-        <v>3.23</v>
+        <v>3.19</v>
       </c>
       <c r="E25" t="n">
-        <v>3.13</v>
+        <v>2.98</v>
       </c>
       <c r="F25" t="n">
-        <v>4.019</v>
+        <v>4.017</v>
       </c>
       <c r="G25" t="n">
-        <v>4.368</v>
+        <v>4.482</v>
       </c>
       <c r="H25" t="n">
-        <v>4.476</v>
+        <v>4.653</v>
       </c>
       <c r="I25" t="n">
-        <v>3.795</v>
+        <v>3.952</v>
       </c>
       <c r="J25" t="n">
         <v>3.64</v>
@@ -1309,32 +1309,32 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="C26" t="n">
-        <v>3.12</v>
+        <v>2.92</v>
       </c>
       <c r="D26" t="n">
-        <v>3.23</v>
+        <v>3.19</v>
       </c>
       <c r="E26" t="n">
-        <v>3.13</v>
+        <v>2.98</v>
       </c>
       <c r="F26" t="n">
-        <v>4.019</v>
+        <v>3.996</v>
       </c>
       <c r="G26" t="n">
-        <v>4.368</v>
+        <v>4.414</v>
       </c>
       <c r="H26" t="n">
-        <v>4.476</v>
+        <v>4.57</v>
       </c>
       <c r="I26" t="n">
-        <v>3.795</v>
+        <v>3.867</v>
       </c>
       <c r="J26" t="n">
         <v>3.64</v>
@@ -1343,32 +1343,32 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="C27" t="n">
-        <v>3.12</v>
+        <v>2.92</v>
       </c>
       <c r="D27" t="n">
-        <v>3.23</v>
+        <v>3.19</v>
       </c>
       <c r="E27" t="n">
-        <v>3.13</v>
+        <v>2.98</v>
       </c>
       <c r="F27" t="n">
-        <v>4.019</v>
+        <v>3.987</v>
       </c>
       <c r="G27" t="n">
-        <v>4.368</v>
+        <v>4.386</v>
       </c>
       <c r="H27" t="n">
-        <v>4.476</v>
+        <v>4.532</v>
       </c>
       <c r="I27" t="n">
-        <v>3.795</v>
+        <v>3.83</v>
       </c>
       <c r="J27" t="n">
         <v>3.64</v>
@@ -1377,32 +1377,32 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="C28" t="n">
-        <v>3.12</v>
+        <v>2.92</v>
       </c>
       <c r="D28" t="n">
-        <v>3.23</v>
+        <v>3.19</v>
       </c>
       <c r="E28" t="n">
-        <v>3.13</v>
+        <v>2.98</v>
       </c>
       <c r="F28" t="n">
-        <v>4.028</v>
+        <v>3.981</v>
       </c>
       <c r="G28" t="n">
-        <v>4.402</v>
+        <v>4.371</v>
       </c>
       <c r="H28" t="n">
-        <v>4.519</v>
+        <v>4.505</v>
       </c>
       <c r="I28" t="n">
-        <v>3.84</v>
+        <v>3.803</v>
       </c>
       <c r="J28" t="n">
         <v>3.65</v>
@@ -1411,100 +1411,100 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="C29" t="n">
-        <v>3.12</v>
+        <v>2.92</v>
       </c>
       <c r="D29" t="n">
-        <v>3.23</v>
+        <v>3.19</v>
       </c>
       <c r="E29" t="n">
-        <v>3.14</v>
+        <v>2.98</v>
       </c>
       <c r="F29" t="n">
-        <v>4.041</v>
+        <v>3.991</v>
       </c>
       <c r="G29" t="n">
-        <v>4.433</v>
+        <v>4.386</v>
       </c>
       <c r="H29" t="n">
-        <v>4.557</v>
+        <v>4.528</v>
       </c>
       <c r="I29" t="n">
-        <v>3.878</v>
+        <v>3.827</v>
       </c>
       <c r="J29" t="n">
-        <v>3.68</v>
+        <v>3.65</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="C30" t="n">
-        <v>3.12</v>
+        <v>2.95</v>
       </c>
       <c r="D30" t="n">
-        <v>3.23</v>
+        <v>3.19</v>
       </c>
       <c r="E30" t="n">
-        <v>3.15</v>
+        <v>2.98</v>
       </c>
       <c r="F30" t="n">
-        <v>4.049</v>
+        <v>3.974</v>
       </c>
       <c r="G30" t="n">
-        <v>4.469</v>
+        <v>4.347</v>
       </c>
       <c r="H30" t="n">
-        <v>4.612</v>
+        <v>4.461</v>
       </c>
       <c r="I30" t="n">
-        <v>3.935</v>
+        <v>3.76</v>
       </c>
       <c r="J30" t="n">
-        <v>3.66</v>
+        <v>3.65</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="C31" t="n">
-        <v>3.12</v>
+        <v>2.95</v>
       </c>
       <c r="D31" t="n">
-        <v>3.24</v>
+        <v>3.19</v>
       </c>
       <c r="E31" t="n">
-        <v>3.16</v>
+        <v>2.98</v>
       </c>
       <c r="F31" t="n">
-        <v>4.046</v>
+        <v>3.974</v>
       </c>
       <c r="G31" t="n">
-        <v>4.417</v>
+        <v>4.347</v>
       </c>
       <c r="H31" t="n">
-        <v>4.558</v>
+        <v>4.461</v>
       </c>
       <c r="I31" t="n">
-        <v>3.882</v>
+        <v>3.76</v>
       </c>
       <c r="J31" t="n">
         <v>3.65</v>
@@ -1513,66 +1513,66 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="C32" t="n">
-        <v>3.12</v>
+        <v>2.95</v>
       </c>
       <c r="D32" t="n">
-        <v>3.24</v>
+        <v>3.19</v>
       </c>
       <c r="E32" t="n">
-        <v>3.16</v>
+        <v>2.98</v>
       </c>
       <c r="F32" t="n">
-        <v>4.048</v>
+        <v>3.974</v>
       </c>
       <c r="G32" t="n">
-        <v>4.411</v>
+        <v>4.347</v>
       </c>
       <c r="H32" t="n">
-        <v>4.558</v>
+        <v>4.461</v>
       </c>
       <c r="I32" t="n">
-        <v>3.885</v>
+        <v>3.76</v>
       </c>
       <c r="J32" t="n">
-        <v>3.66</v>
+        <v>3.65</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="C33" t="n">
-        <v>3.12</v>
+        <v>2.93</v>
       </c>
       <c r="D33" t="n">
-        <v>3.24</v>
+        <v>3.19</v>
       </c>
       <c r="E33" t="n">
-        <v>3.16</v>
+        <v>2.98</v>
       </c>
       <c r="F33" t="n">
-        <v>4.048</v>
+        <v>3.964</v>
       </c>
       <c r="G33" t="n">
-        <v>4.411</v>
+        <v>4.331</v>
       </c>
       <c r="H33" t="n">
-        <v>4.558</v>
+        <v>4.443</v>
       </c>
       <c r="I33" t="n">
-        <v>3.885</v>
+        <v>3.742</v>
       </c>
       <c r="J33" t="n">
         <v>3.66</v>
@@ -1581,66 +1581,66 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="C34" t="n">
-        <v>3.12</v>
+        <v>2.93</v>
       </c>
       <c r="D34" t="n">
-        <v>3.24</v>
+        <v>3.19</v>
       </c>
       <c r="E34" t="n">
-        <v>3.16</v>
+        <v>2.98</v>
       </c>
       <c r="F34" t="n">
-        <v>4.048</v>
+        <v>3.962</v>
       </c>
       <c r="G34" t="n">
-        <v>4.411</v>
+        <v>4.343</v>
       </c>
       <c r="H34" t="n">
-        <v>4.558</v>
+        <v>4.441</v>
       </c>
       <c r="I34" t="n">
-        <v>3.885</v>
+        <v>3.74</v>
       </c>
       <c r="J34" t="n">
-        <v>3.66</v>
+        <v>3.65</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="C35" t="n">
-        <v>3.12</v>
+        <v>2.93</v>
       </c>
       <c r="D35" t="n">
-        <v>3.24</v>
+        <v>3.19</v>
       </c>
       <c r="E35" t="n">
-        <v>3.16</v>
+        <v>2.98</v>
       </c>
       <c r="F35" t="n">
-        <v>4.054</v>
+        <v>3.943</v>
       </c>
       <c r="G35" t="n">
-        <v>4.43</v>
+        <v>4.273</v>
       </c>
       <c r="H35" t="n">
-        <v>4.57</v>
+        <v>4.38</v>
       </c>
       <c r="I35" t="n">
-        <v>3.897</v>
+        <v>3.677</v>
       </c>
       <c r="J35" t="n">
         <v>3.66</v>
@@ -1649,102 +1649,1224 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="C36" t="n">
-        <v>3.12</v>
+        <v>2.93</v>
       </c>
       <c r="D36" t="n">
-        <v>3.25</v>
+        <v>3.19</v>
       </c>
       <c r="E36" t="n">
-        <v>3.17</v>
+        <v>2.98</v>
       </c>
       <c r="F36" t="n">
-        <v>4.069</v>
+        <v>3.946</v>
       </c>
       <c r="G36" t="n">
-        <v>4.438</v>
+        <v>4.308</v>
       </c>
       <c r="H36" t="n">
-        <v>4.568</v>
+        <v>4.441</v>
       </c>
       <c r="I36" t="n">
-        <v>3.897</v>
+        <v>3.745</v>
       </c>
       <c r="J36" t="n">
-        <v>3.65</v>
+        <v>3.64</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="C37" t="n">
-        <v>3.12</v>
+        <v>2.93</v>
       </c>
       <c r="D37" t="n">
-        <v>3.25</v>
+        <v>3.19</v>
       </c>
       <c r="E37" t="n">
-        <v>3.18</v>
+        <v>2.99</v>
       </c>
       <c r="F37" t="n">
-        <v>4.078</v>
+        <v>3.944</v>
       </c>
       <c r="G37" t="n">
-        <v>4.445</v>
+        <v>4.308</v>
       </c>
       <c r="H37" t="n">
-        <v>4.58</v>
+        <v>4.441</v>
       </c>
       <c r="I37" t="n">
-        <v>3.91</v>
+        <v>3.747</v>
       </c>
       <c r="J37" t="n">
-        <v>3.64</v>
+        <v>3.65</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C38" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D38" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E38" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="F38" t="n">
+        <v>3.944</v>
+      </c>
+      <c r="G38" t="n">
+        <v>4.308</v>
+      </c>
+      <c r="H38" t="n">
+        <v>4.441</v>
+      </c>
+      <c r="I38" t="n">
+        <v>3.747</v>
+      </c>
+      <c r="J38" t="n">
+        <v>3.65</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C39" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D39" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E39" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="F39" t="n">
+        <v>3.944</v>
+      </c>
+      <c r="G39" t="n">
+        <v>4.308</v>
+      </c>
+      <c r="H39" t="n">
+        <v>4.441</v>
+      </c>
+      <c r="I39" t="n">
+        <v>3.747</v>
+      </c>
+      <c r="J39" t="n">
+        <v>3.65</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C40" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D40" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E40" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="F40" t="n">
+        <v>3.958</v>
+      </c>
+      <c r="G40" t="n">
+        <v>4.324</v>
+      </c>
+      <c r="H40" t="n">
+        <v>4.465</v>
+      </c>
+      <c r="I40" t="n">
+        <v>3.775</v>
+      </c>
+      <c r="J40" t="n">
+        <v>3.62</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C41" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D41" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E41" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="F41" t="n">
+        <v>3.971</v>
+      </c>
+      <c r="G41" t="n">
+        <v>4.357</v>
+      </c>
+      <c r="H41" t="n">
+        <v>4.486</v>
+      </c>
+      <c r="I41" t="n">
+        <v>3.797</v>
+      </c>
+      <c r="J41" t="n">
+        <v>3.63</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C42" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D42" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E42" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="F42" t="n">
+        <v>3.962</v>
+      </c>
+      <c r="G42" t="n">
+        <v>4.341</v>
+      </c>
+      <c r="H42" t="n">
+        <v>4.471</v>
+      </c>
+      <c r="I42" t="n">
+        <v>3.782</v>
+      </c>
+      <c r="J42" t="n">
+        <v>3.64</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C43" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D43" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E43" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="F43" t="n">
+        <v>3.961</v>
+      </c>
+      <c r="G43" t="n">
+        <v>4.348</v>
+      </c>
+      <c r="H43" t="n">
+        <v>4.464</v>
+      </c>
+      <c r="I43" t="n">
+        <v>3.777</v>
+      </c>
+      <c r="J43" t="n">
+        <v>3.62</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C44" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D44" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E44" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="F44" t="n">
+        <v>3.949</v>
+      </c>
+      <c r="G44" t="n">
+        <v>4.357</v>
+      </c>
+      <c r="H44" t="n">
+        <v>4.477</v>
+      </c>
+      <c r="I44" t="n">
+        <v>3.795</v>
+      </c>
+      <c r="J44" t="n">
+        <v>3.62</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C45" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D45" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E45" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="F45" t="n">
+        <v>3.949</v>
+      </c>
+      <c r="G45" t="n">
+        <v>4.357</v>
+      </c>
+      <c r="H45" t="n">
+        <v>4.477</v>
+      </c>
+      <c r="I45" t="n">
+        <v>3.795</v>
+      </c>
+      <c r="J45" t="n">
+        <v>3.62</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C46" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D46" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E46" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="F46" t="n">
+        <v>3.949</v>
+      </c>
+      <c r="G46" t="n">
+        <v>4.357</v>
+      </c>
+      <c r="H46" t="n">
+        <v>4.477</v>
+      </c>
+      <c r="I46" t="n">
+        <v>3.795</v>
+      </c>
+      <c r="J46" t="n">
+        <v>3.62</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C47" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D47" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E47" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="F47" t="n">
+        <v>3.949</v>
+      </c>
+      <c r="G47" t="n">
+        <v>4.357</v>
+      </c>
+      <c r="H47" t="n">
+        <v>4.477</v>
+      </c>
+      <c r="I47" t="n">
+        <v>3.795</v>
+      </c>
+      <c r="J47" t="n">
+        <v>3.62</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C48" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D48" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E48" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="F48" t="n">
+        <v>3.968</v>
+      </c>
+      <c r="G48" t="n">
+        <v>4.397</v>
+      </c>
+      <c r="H48" t="n">
+        <v>4.522</v>
+      </c>
+      <c r="I48" t="n">
+        <v>3.84</v>
+      </c>
+      <c r="J48" t="n">
+        <v>3.66</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C49" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D49" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E49" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="F49" t="n">
+        <v>3.969</v>
+      </c>
+      <c r="G49" t="n">
+        <v>4.355</v>
+      </c>
+      <c r="H49" t="n">
+        <v>4.471</v>
+      </c>
+      <c r="I49" t="n">
+        <v>3.787</v>
+      </c>
+      <c r="J49" t="n">
+        <v>3.65</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C50" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D50" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E50" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="F50" t="n">
+        <v>3.984</v>
+      </c>
+      <c r="G50" t="n">
+        <v>4.391</v>
+      </c>
+      <c r="H50" t="n">
+        <v>4.503</v>
+      </c>
+      <c r="I50" t="n">
+        <v>3.822</v>
+      </c>
+      <c r="J50" t="n">
+        <v>3.62</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C51" t="n">
+        <v>2.94</v>
+      </c>
+      <c r="D51" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E51" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="F51" t="n">
+        <v>4.004</v>
+      </c>
+      <c r="G51" t="n">
+        <v>4.414</v>
+      </c>
+      <c r="H51" t="n">
+        <v>4.535</v>
+      </c>
+      <c r="I51" t="n">
+        <v>3.855</v>
+      </c>
+      <c r="J51" t="n">
+        <v>3.63</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C52" t="n">
+        <v>2.94</v>
+      </c>
+      <c r="D52" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E52" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="F52" t="n">
+        <v>4.004</v>
+      </c>
+      <c r="G52" t="n">
+        <v>4.414</v>
+      </c>
+      <c r="H52" t="n">
+        <v>4.535</v>
+      </c>
+      <c r="I52" t="n">
+        <v>3.855</v>
+      </c>
+      <c r="J52" t="n">
+        <v>3.63</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C53" t="n">
+        <v>2.94</v>
+      </c>
+      <c r="D53" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E53" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="F53" t="n">
+        <v>4.004</v>
+      </c>
+      <c r="G53" t="n">
+        <v>4.414</v>
+      </c>
+      <c r="H53" t="n">
+        <v>4.535</v>
+      </c>
+      <c r="I53" t="n">
+        <v>3.855</v>
+      </c>
+      <c r="J53" t="n">
+        <v>3.63</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C54" t="n">
+        <v>2.95</v>
+      </c>
+      <c r="D54" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E54" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="F54" t="n">
+        <v>4.006</v>
+      </c>
+      <c r="G54" t="n">
+        <v>4.396</v>
+      </c>
+      <c r="H54" t="n">
+        <v>4.516</v>
+      </c>
+      <c r="I54" t="n">
+        <v>3.835</v>
+      </c>
+      <c r="J54" t="n">
+        <v>3.65</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C55" t="n">
+        <v>2.95</v>
+      </c>
+      <c r="D55" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E55" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="F55" t="n">
+        <v>4.013</v>
+      </c>
+      <c r="G55" t="n">
+        <v>4.383</v>
+      </c>
+      <c r="H55" t="n">
+        <v>4.508</v>
+      </c>
+      <c r="I55" t="n">
+        <v>3.826</v>
+      </c>
+      <c r="J55" t="n">
+        <v>3.65</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C56" t="n">
+        <v>2.96</v>
+      </c>
+      <c r="D56" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="E56" t="n">
+        <v>3</v>
+      </c>
+      <c r="F56" t="n">
+        <v>4.019</v>
+      </c>
+      <c r="G56" t="n">
+        <v>4.384</v>
+      </c>
+      <c r="H56" t="n">
+        <v>4.498</v>
+      </c>
+      <c r="I56" t="n">
+        <v>3.817</v>
+      </c>
+      <c r="J56" t="n">
+        <v>3.66</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>3</v>
+      </c>
+      <c r="C57" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="D57" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="E57" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="F57" t="n">
+        <v>4.014</v>
+      </c>
+      <c r="G57" t="n">
+        <v>4.322</v>
+      </c>
+      <c r="H57" t="n">
+        <v>4.433</v>
+      </c>
+      <c r="I57" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="J57" t="n">
+        <v>3.64</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>3</v>
+      </c>
+      <c r="C58" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="D58" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="E58" t="n">
+        <v>3.13</v>
+      </c>
+      <c r="F58" t="n">
+        <v>4.019</v>
+      </c>
+      <c r="G58" t="n">
+        <v>4.368</v>
+      </c>
+      <c r="H58" t="n">
+        <v>4.476</v>
+      </c>
+      <c r="I58" t="n">
+        <v>3.795</v>
+      </c>
+      <c r="J58" t="n">
+        <v>3.64</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>3</v>
+      </c>
+      <c r="C59" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="D59" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="E59" t="n">
+        <v>3.13</v>
+      </c>
+      <c r="F59" t="n">
+        <v>4.019</v>
+      </c>
+      <c r="G59" t="n">
+        <v>4.368</v>
+      </c>
+      <c r="H59" t="n">
+        <v>4.476</v>
+      </c>
+      <c r="I59" t="n">
+        <v>3.795</v>
+      </c>
+      <c r="J59" t="n">
+        <v>3.64</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>3</v>
+      </c>
+      <c r="C60" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="D60" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="E60" t="n">
+        <v>3.13</v>
+      </c>
+      <c r="F60" t="n">
+        <v>4.019</v>
+      </c>
+      <c r="G60" t="n">
+        <v>4.368</v>
+      </c>
+      <c r="H60" t="n">
+        <v>4.476</v>
+      </c>
+      <c r="I60" t="n">
+        <v>3.795</v>
+      </c>
+      <c r="J60" t="n">
+        <v>3.64</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>3</v>
+      </c>
+      <c r="C61" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="D61" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="E61" t="n">
+        <v>3.13</v>
+      </c>
+      <c r="F61" t="n">
+        <v>4.028</v>
+      </c>
+      <c r="G61" t="n">
+        <v>4.402</v>
+      </c>
+      <c r="H61" t="n">
+        <v>4.519</v>
+      </c>
+      <c r="I61" t="n">
+        <v>3.84</v>
+      </c>
+      <c r="J61" t="n">
+        <v>3.65</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>3</v>
+      </c>
+      <c r="C62" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="D62" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="E62" t="n">
+        <v>3.14</v>
+      </c>
+      <c r="F62" t="n">
+        <v>4.041</v>
+      </c>
+      <c r="G62" t="n">
+        <v>4.433</v>
+      </c>
+      <c r="H62" t="n">
+        <v>4.557</v>
+      </c>
+      <c r="I62" t="n">
+        <v>3.878</v>
+      </c>
+      <c r="J62" t="n">
+        <v>3.68</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>3</v>
+      </c>
+      <c r="C63" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="D63" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="E63" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="F63" t="n">
+        <v>4.049</v>
+      </c>
+      <c r="G63" t="n">
+        <v>4.469</v>
+      </c>
+      <c r="H63" t="n">
+        <v>4.612</v>
+      </c>
+      <c r="I63" t="n">
+        <v>3.935</v>
+      </c>
+      <c r="J63" t="n">
+        <v>3.66</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>3</v>
+      </c>
+      <c r="C64" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="D64" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="E64" t="n">
+        <v>3.16</v>
+      </c>
+      <c r="F64" t="n">
+        <v>4.046</v>
+      </c>
+      <c r="G64" t="n">
+        <v>4.417</v>
+      </c>
+      <c r="H64" t="n">
+        <v>4.558</v>
+      </c>
+      <c r="I64" t="n">
+        <v>3.882</v>
+      </c>
+      <c r="J64" t="n">
+        <v>3.65</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>3</v>
+      </c>
+      <c r="C65" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="D65" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="E65" t="n">
+        <v>3.16</v>
+      </c>
+      <c r="F65" t="n">
+        <v>4.048</v>
+      </c>
+      <c r="G65" t="n">
+        <v>4.411</v>
+      </c>
+      <c r="H65" t="n">
+        <v>4.558</v>
+      </c>
+      <c r="I65" t="n">
+        <v>3.885</v>
+      </c>
+      <c r="J65" t="n">
+        <v>3.66</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>3</v>
+      </c>
+      <c r="C66" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="D66" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="E66" t="n">
+        <v>3.16</v>
+      </c>
+      <c r="F66" t="n">
+        <v>4.048</v>
+      </c>
+      <c r="G66" t="n">
+        <v>4.411</v>
+      </c>
+      <c r="H66" t="n">
+        <v>4.558</v>
+      </c>
+      <c r="I66" t="n">
+        <v>3.885</v>
+      </c>
+      <c r="J66" t="n">
+        <v>3.66</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>3</v>
+      </c>
+      <c r="C67" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="D67" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="E67" t="n">
+        <v>3.16</v>
+      </c>
+      <c r="F67" t="n">
+        <v>4.048</v>
+      </c>
+      <c r="G67" t="n">
+        <v>4.411</v>
+      </c>
+      <c r="H67" t="n">
+        <v>4.558</v>
+      </c>
+      <c r="I67" t="n">
+        <v>3.885</v>
+      </c>
+      <c r="J67" t="n">
+        <v>3.66</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>3</v>
+      </c>
+      <c r="C68" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="D68" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="E68" t="n">
+        <v>3.16</v>
+      </c>
+      <c r="F68" t="n">
+        <v>4.054</v>
+      </c>
+      <c r="G68" t="n">
+        <v>4.43</v>
+      </c>
+      <c r="H68" t="n">
+        <v>4.57</v>
+      </c>
+      <c r="I68" t="n">
+        <v>3.897</v>
+      </c>
+      <c r="J68" t="n">
+        <v>3.65</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>3</v>
+      </c>
+      <c r="C69" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="D69" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="E69" t="n">
+        <v>3.17</v>
+      </c>
+      <c r="F69" t="n">
+        <v>4.069</v>
+      </c>
+      <c r="G69" t="n">
+        <v>4.438</v>
+      </c>
+      <c r="H69" t="n">
+        <v>4.568</v>
+      </c>
+      <c r="I69" t="n">
+        <v>3.897</v>
+      </c>
+      <c r="J69" t="n">
+        <v>3.65</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>3</v>
+      </c>
+      <c r="C70" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="D70" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="E70" t="n">
+        <v>3.18</v>
+      </c>
+      <c r="F70" t="n">
+        <v>4.078</v>
+      </c>
+      <c r="G70" t="n">
+        <v>4.445</v>
+      </c>
+      <c r="H70" t="n">
+        <v>4.58</v>
+      </c>
+      <c r="I70" t="n">
+        <v>3.91</v>
+      </c>
+      <c r="J70" t="n">
+        <v>3.64</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
           <t>2026-09-10</t>
         </is>
       </c>
-      <c r="B38" t="n">
+      <c r="B71" t="n">
         <v>3</v>
       </c>
-      <c r="C38" t="n">
+      <c r="C71" t="n">
         <v>3.12</v>
       </c>
-      <c r="D38" t="n">
+      <c r="D71" t="n">
         <v>3.26</v>
       </c>
-      <c r="E38" t="n">
+      <c r="E71" t="n">
         <v>3.18</v>
       </c>
-      <c r="F38" t="n">
+      <c r="F71" t="n">
         <v>4.091</v>
       </c>
-      <c r="G38" t="n">
+      <c r="G71" t="n">
         <v>4.464</v>
       </c>
-      <c r="H38" t="n">
+      <c r="H71" t="n">
         <v>4.595</v>
       </c>
-      <c r="I38" t="n">
+      <c r="I71" t="n">
         <v>3.927</v>
       </c>
-      <c r="J38" t="n">
+      <c r="J71" t="n">
         <v>3.64</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: backfill rates (80 business days)
</commit_message>
<xml_diff>
--- a/docs/data/history.xlsx
+++ b/docs/data/history.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J71"/>
+  <dimension ref="A1:J113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -493,440 +493,440 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B2" t="n">
         <v>2.5</v>
       </c>
       <c r="C2" t="n">
-        <v>2.92</v>
+        <v>2.81</v>
       </c>
       <c r="D2" t="n">
-        <v>3.19</v>
+        <v>3.05</v>
       </c>
       <c r="E2" t="n">
-        <v>2.96</v>
+        <v>2.86</v>
       </c>
       <c r="F2" t="n">
-        <v>3.973</v>
+        <v>3.588</v>
       </c>
       <c r="G2" t="n">
-        <v>4.4</v>
+        <v>4.165</v>
       </c>
       <c r="H2" t="n">
-        <v>4.437</v>
+        <v>4.341</v>
       </c>
       <c r="I2" t="n">
-        <v>3.745</v>
+        <v>3.725</v>
       </c>
       <c r="J2" t="n">
-        <v>3.64</v>
+        <v>3.51</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B3" t="n">
         <v>2.5</v>
       </c>
       <c r="C3" t="n">
-        <v>2.92</v>
+        <v>2.81</v>
       </c>
       <c r="D3" t="n">
-        <v>3.19</v>
+        <v>3.05</v>
       </c>
       <c r="E3" t="n">
-        <v>2.96</v>
+        <v>2.86</v>
       </c>
       <c r="F3" t="n">
-        <v>3.973</v>
+        <v>3.588</v>
       </c>
       <c r="G3" t="n">
-        <v>4.4</v>
+        <v>4.165</v>
       </c>
       <c r="H3" t="n">
-        <v>4.437</v>
+        <v>4.341</v>
       </c>
       <c r="I3" t="n">
-        <v>3.745</v>
+        <v>3.725</v>
       </c>
       <c r="J3" t="n">
-        <v>3.64</v>
+        <v>3.55</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B4" t="n">
         <v>2.5</v>
       </c>
       <c r="C4" t="n">
-        <v>2.92</v>
+        <v>2.81</v>
       </c>
       <c r="D4" t="n">
-        <v>3.19</v>
+        <v>3.05</v>
       </c>
       <c r="E4" t="n">
-        <v>2.96</v>
+        <v>2.86</v>
       </c>
       <c r="F4" t="n">
-        <v>3.973</v>
+        <v>3.588</v>
       </c>
       <c r="G4" t="n">
-        <v>4.4</v>
+        <v>4.165</v>
       </c>
       <c r="H4" t="n">
-        <v>4.437</v>
+        <v>4.341</v>
       </c>
       <c r="I4" t="n">
-        <v>3.745</v>
+        <v>3.725</v>
       </c>
       <c r="J4" t="n">
-        <v>3.64</v>
+        <v>3.55</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>2.5</v>
       </c>
       <c r="C5" t="n">
-        <v>2.92</v>
+        <v>2.81</v>
       </c>
       <c r="D5" t="n">
-        <v>3.19</v>
+        <v>3.05</v>
       </c>
       <c r="E5" t="n">
-        <v>2.95</v>
+        <v>2.86</v>
       </c>
       <c r="F5" t="n">
-        <v>3.976</v>
+        <v>3.588</v>
       </c>
       <c r="G5" t="n">
-        <v>4.401</v>
+        <v>4.165</v>
       </c>
       <c r="H5" t="n">
-        <v>4.461</v>
+        <v>4.341</v>
       </c>
       <c r="I5" t="n">
-        <v>3.77</v>
+        <v>3.725</v>
       </c>
       <c r="J5" t="n">
-        <v>3.64</v>
+        <v>3.55</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>2.5</v>
       </c>
       <c r="C6" t="n">
-        <v>2.91</v>
+        <v>2.82</v>
       </c>
       <c r="D6" t="n">
-        <v>3.18</v>
+        <v>3.06</v>
       </c>
       <c r="E6" t="n">
-        <v>2.94</v>
+        <v>2.86</v>
       </c>
       <c r="F6" t="n">
-        <v>3.977</v>
+        <v>3.607</v>
       </c>
       <c r="G6" t="n">
-        <v>4.399</v>
+        <v>4.112</v>
       </c>
       <c r="H6" t="n">
-        <v>4.469</v>
+        <v>4.281</v>
       </c>
       <c r="I6" t="n">
-        <v>3.777</v>
+        <v>3.664</v>
       </c>
       <c r="J6" t="n">
-        <v>3.63</v>
+        <v>3.55</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>2.5</v>
       </c>
       <c r="C7" t="n">
-        <v>2.91</v>
+        <v>2.83</v>
       </c>
       <c r="D7" t="n">
-        <v>3.18</v>
+        <v>3.06</v>
       </c>
       <c r="E7" t="n">
-        <v>2.94</v>
+        <v>2.86</v>
       </c>
       <c r="F7" t="n">
-        <v>3.986</v>
+        <v>3.648</v>
       </c>
       <c r="G7" t="n">
-        <v>4.395</v>
+        <v>4.158</v>
       </c>
       <c r="H7" t="n">
-        <v>4.472</v>
+        <v>4.333</v>
       </c>
       <c r="I7" t="n">
-        <v>3.776</v>
+        <v>3.717</v>
       </c>
       <c r="J7" t="n">
-        <v>3.62</v>
+        <v>3.63</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>2.5</v>
       </c>
       <c r="C8" t="n">
-        <v>2.91</v>
+        <v>2.85</v>
       </c>
       <c r="D8" t="n">
-        <v>3.18</v>
+        <v>3.06</v>
       </c>
       <c r="E8" t="n">
-        <v>2.93</v>
+        <v>2.86</v>
       </c>
       <c r="F8" t="n">
-        <v>3.991</v>
+        <v>3.685</v>
       </c>
       <c r="G8" t="n">
-        <v>4.407</v>
+        <v>4.211</v>
       </c>
       <c r="H8" t="n">
-        <v>4.478</v>
+        <v>4.383</v>
       </c>
       <c r="I8" t="n">
-        <v>3.78</v>
+        <v>3.767</v>
       </c>
       <c r="J8" t="n">
-        <v>3.58</v>
+        <v>3.63</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B9" t="n">
         <v>2.5</v>
       </c>
       <c r="C9" t="n">
-        <v>2.9</v>
+        <v>2.85</v>
       </c>
       <c r="D9" t="n">
-        <v>3.17</v>
+        <v>3.07</v>
       </c>
       <c r="E9" t="n">
-        <v>2.93</v>
+        <v>2.86</v>
       </c>
       <c r="F9" t="n">
-        <v>3.997</v>
+        <v>3.683</v>
       </c>
       <c r="G9" t="n">
-        <v>4.399</v>
+        <v>4.208</v>
       </c>
       <c r="H9" t="n">
-        <v>4.47</v>
+        <v>4.34</v>
       </c>
       <c r="I9" t="n">
-        <v>3.77</v>
+        <v>3.722</v>
       </c>
       <c r="J9" t="n">
-        <v>3.53</v>
+        <v>3.62</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B10" t="n">
         <v>2.5</v>
       </c>
       <c r="C10" t="n">
-        <v>2.9</v>
+        <v>2.85</v>
       </c>
       <c r="D10" t="n">
-        <v>3.17</v>
+        <v>3.07</v>
       </c>
       <c r="E10" t="n">
-        <v>2.93</v>
+        <v>2.86</v>
       </c>
       <c r="F10" t="n">
-        <v>3.997</v>
+        <v>3.683</v>
       </c>
       <c r="G10" t="n">
-        <v>4.399</v>
+        <v>4.208</v>
       </c>
       <c r="H10" t="n">
-        <v>4.47</v>
+        <v>4.34</v>
       </c>
       <c r="I10" t="n">
-        <v>3.77</v>
+        <v>3.722</v>
       </c>
       <c r="J10" t="n">
-        <v>3.53</v>
+        <v>3.63</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>2.5</v>
       </c>
       <c r="C11" t="n">
-        <v>2.9</v>
+        <v>2.85</v>
       </c>
       <c r="D11" t="n">
-        <v>3.17</v>
+        <v>3.07</v>
       </c>
       <c r="E11" t="n">
-        <v>2.93</v>
+        <v>2.86</v>
       </c>
       <c r="F11" t="n">
-        <v>3.997</v>
+        <v>3.683</v>
       </c>
       <c r="G11" t="n">
-        <v>4.399</v>
+        <v>4.208</v>
       </c>
       <c r="H11" t="n">
-        <v>4.47</v>
+        <v>4.34</v>
       </c>
       <c r="I11" t="n">
-        <v>3.77</v>
+        <v>3.722</v>
       </c>
       <c r="J11" t="n">
-        <v>3.53</v>
+        <v>3.63</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B12" t="n">
         <v>2.5</v>
       </c>
       <c r="C12" t="n">
-        <v>2.9</v>
+        <v>2.85</v>
       </c>
       <c r="D12" t="n">
-        <v>3.17</v>
+        <v>3.07</v>
       </c>
       <c r="E12" t="n">
-        <v>2.92</v>
+        <v>2.87</v>
       </c>
       <c r="F12" t="n">
-        <v>4.009</v>
+        <v>3.697</v>
       </c>
       <c r="G12" t="n">
-        <v>4.429</v>
+        <v>4.261</v>
       </c>
       <c r="H12" t="n">
-        <v>4.513</v>
+        <v>4.406</v>
       </c>
       <c r="I12" t="n">
-        <v>3.81</v>
+        <v>3.79</v>
       </c>
       <c r="J12" t="n">
-        <v>3.55</v>
+        <v>3.63</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B13" t="n">
         <v>2.5</v>
       </c>
       <c r="C13" t="n">
-        <v>2.9</v>
+        <v>2.87</v>
       </c>
       <c r="D13" t="n">
-        <v>3.17</v>
+        <v>3.08</v>
       </c>
       <c r="E13" t="n">
-        <v>2.92</v>
+        <v>2.87</v>
       </c>
       <c r="F13" t="n">
-        <v>4.036</v>
+        <v>3.7</v>
       </c>
       <c r="G13" t="n">
-        <v>4.489</v>
+        <v>4.285</v>
       </c>
       <c r="H13" t="n">
-        <v>4.594</v>
+        <v>4.386</v>
       </c>
       <c r="I13" t="n">
-        <v>3.89</v>
+        <v>3.77</v>
       </c>
       <c r="J13" t="n">
-        <v>3.6</v>
+        <v>3.65</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B14" t="n">
         <v>2.5</v>
       </c>
       <c r="C14" t="n">
-        <v>2.9</v>
+        <v>2.87</v>
       </c>
       <c r="D14" t="n">
-        <v>3.17</v>
+        <v>3.08</v>
       </c>
       <c r="E14" t="n">
-        <v>2.92</v>
+        <v>2.87</v>
       </c>
       <c r="F14" t="n">
-        <v>4.018</v>
+        <v>3.7</v>
       </c>
       <c r="G14" t="n">
-        <v>4.462</v>
+        <v>4.285</v>
       </c>
       <c r="H14" t="n">
-        <v>4.572</v>
+        <v>4.386</v>
       </c>
       <c r="I14" t="n">
-        <v>3.867</v>
+        <v>3.77</v>
       </c>
       <c r="J14" t="n">
         <v>3.63</v>
@@ -935,66 +935,66 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C15" t="n">
-        <v>2.9</v>
+        <v>2.87</v>
       </c>
       <c r="D15" t="n">
-        <v>3.17</v>
+        <v>3.08</v>
       </c>
       <c r="E15" t="n">
-        <v>2.97</v>
+        <v>2.87</v>
       </c>
       <c r="F15" t="n">
-        <v>3.992</v>
+        <v>3.769</v>
       </c>
       <c r="G15" t="n">
-        <v>4.424</v>
+        <v>4.362</v>
       </c>
       <c r="H15" t="n">
-        <v>4.554</v>
+        <v>4.476</v>
       </c>
       <c r="I15" t="n">
-        <v>3.852</v>
+        <v>3.86</v>
       </c>
       <c r="J15" t="n">
-        <v>3.64</v>
+        <v>3.61</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C16" t="n">
-        <v>2.9</v>
+        <v>2.88</v>
       </c>
       <c r="D16" t="n">
-        <v>3.17</v>
+        <v>3.09</v>
       </c>
       <c r="E16" t="n">
-        <v>2.97</v>
+        <v>2.88</v>
       </c>
       <c r="F16" t="n">
-        <v>3.992</v>
+        <v>3.777</v>
       </c>
       <c r="G16" t="n">
-        <v>4.424</v>
+        <v>4.38</v>
       </c>
       <c r="H16" t="n">
-        <v>4.554</v>
+        <v>4.496</v>
       </c>
       <c r="I16" t="n">
-        <v>3.852</v>
+        <v>3.88</v>
       </c>
       <c r="J16" t="n">
         <v>3.62</v>
@@ -1003,814 +1003,814 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C17" t="n">
-        <v>2.9</v>
+        <v>2.88</v>
       </c>
       <c r="D17" t="n">
-        <v>3.17</v>
+        <v>3.09</v>
       </c>
       <c r="E17" t="n">
-        <v>2.97</v>
+        <v>2.88</v>
       </c>
       <c r="F17" t="n">
-        <v>3.992</v>
+        <v>3.777</v>
       </c>
       <c r="G17" t="n">
-        <v>4.424</v>
+        <v>4.38</v>
       </c>
       <c r="H17" t="n">
-        <v>4.554</v>
+        <v>4.496</v>
       </c>
       <c r="I17" t="n">
-        <v>3.852</v>
+        <v>3.88</v>
       </c>
       <c r="J17" t="n">
-        <v>3.62</v>
+        <v>3.63</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C18" t="n">
-        <v>2.9</v>
+        <v>2.88</v>
       </c>
       <c r="D18" t="n">
-        <v>3.17</v>
+        <v>3.09</v>
       </c>
       <c r="E18" t="n">
-        <v>2.97</v>
+        <v>2.88</v>
       </c>
       <c r="F18" t="n">
-        <v>3.992</v>
+        <v>3.777</v>
       </c>
       <c r="G18" t="n">
-        <v>4.424</v>
+        <v>4.38</v>
       </c>
       <c r="H18" t="n">
-        <v>4.554</v>
+        <v>4.496</v>
       </c>
       <c r="I18" t="n">
-        <v>3.852</v>
+        <v>3.88</v>
       </c>
       <c r="J18" t="n">
-        <v>3.62</v>
+        <v>3.63</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C19" t="n">
         <v>2.91</v>
       </c>
       <c r="D19" t="n">
-        <v>3.18</v>
+        <v>3.1</v>
       </c>
       <c r="E19" t="n">
-        <v>2.98</v>
+        <v>2.89</v>
       </c>
       <c r="F19" t="n">
-        <v>4.003</v>
+        <v>3.815</v>
       </c>
       <c r="G19" t="n">
-        <v>4.452</v>
+        <v>4.447</v>
       </c>
       <c r="H19" t="n">
-        <v>4.599</v>
+        <v>4.547</v>
       </c>
       <c r="I19" t="n">
-        <v>3.897</v>
+        <v>3.93</v>
       </c>
       <c r="J19" t="n">
-        <v>3.59</v>
+        <v>3.63</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C20" t="n">
-        <v>2.91</v>
+        <v>2.9</v>
       </c>
       <c r="D20" t="n">
-        <v>3.19</v>
+        <v>3.11</v>
       </c>
       <c r="E20" t="n">
-        <v>2.98</v>
+        <v>2.89</v>
       </c>
       <c r="F20" t="n">
-        <v>3.988</v>
+        <v>3.802</v>
       </c>
       <c r="G20" t="n">
-        <v>4.398</v>
+        <v>4.382</v>
       </c>
       <c r="H20" t="n">
-        <v>4.57</v>
+        <v>4.489</v>
       </c>
       <c r="I20" t="n">
-        <v>3.866</v>
+        <v>3.86</v>
       </c>
       <c r="J20" t="n">
-        <v>3.57</v>
+        <v>3.63</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C21" t="n">
-        <v>2.91</v>
+        <v>2.92</v>
       </c>
       <c r="D21" t="n">
-        <v>3.19</v>
+        <v>3.11</v>
       </c>
       <c r="E21" t="n">
-        <v>2.98</v>
+        <v>2.89</v>
       </c>
       <c r="F21" t="n">
-        <v>3.999</v>
+        <v>3.795</v>
       </c>
       <c r="G21" t="n">
-        <v>4.444</v>
+        <v>4.378</v>
       </c>
       <c r="H21" t="n">
-        <v>4.617</v>
+        <v>4.474</v>
       </c>
       <c r="I21" t="n">
-        <v>3.915</v>
+        <v>3.877</v>
       </c>
       <c r="J21" t="n">
-        <v>3.61</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C22" t="n">
-        <v>2.91</v>
+        <v>2.92</v>
       </c>
       <c r="D22" t="n">
-        <v>3.19</v>
+        <v>3.14</v>
       </c>
       <c r="E22" t="n">
-        <v>2.98</v>
+        <v>2.92</v>
       </c>
       <c r="F22" t="n">
-        <v>4.007</v>
+        <v>3.791</v>
       </c>
       <c r="G22" t="n">
-        <v>4.454</v>
+        <v>4.403</v>
       </c>
       <c r="H22" t="n">
-        <v>4.617</v>
+        <v>4.505</v>
       </c>
       <c r="I22" t="n">
-        <v>3.917</v>
+        <v>3.906</v>
       </c>
       <c r="J22" t="n">
-        <v>3.62</v>
+        <v>3.59</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C23" t="n">
-        <v>2.91</v>
+        <v>2.92</v>
       </c>
       <c r="D23" t="n">
-        <v>3.19</v>
+        <v>3.14</v>
       </c>
       <c r="E23" t="n">
-        <v>2.98</v>
+        <v>2.92</v>
       </c>
       <c r="F23" t="n">
-        <v>4.017</v>
+        <v>3.757</v>
       </c>
       <c r="G23" t="n">
-        <v>4.482</v>
+        <v>4.329</v>
       </c>
       <c r="H23" t="n">
-        <v>4.653</v>
+        <v>4.403</v>
       </c>
       <c r="I23" t="n">
-        <v>3.952</v>
+        <v>3.79</v>
       </c>
       <c r="J23" t="n">
-        <v>3.64</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C24" t="n">
-        <v>2.91</v>
+        <v>2.92</v>
       </c>
       <c r="D24" t="n">
-        <v>3.19</v>
+        <v>3.14</v>
       </c>
       <c r="E24" t="n">
-        <v>2.98</v>
+        <v>2.92</v>
       </c>
       <c r="F24" t="n">
-        <v>4.017</v>
+        <v>3.757</v>
       </c>
       <c r="G24" t="n">
-        <v>4.482</v>
+        <v>4.329</v>
       </c>
       <c r="H24" t="n">
-        <v>4.653</v>
+        <v>4.403</v>
       </c>
       <c r="I24" t="n">
-        <v>3.952</v>
+        <v>3.79</v>
       </c>
       <c r="J24" t="n">
-        <v>3.64</v>
+        <v>3.65</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C25" t="n">
-        <v>2.91</v>
+        <v>2.92</v>
       </c>
       <c r="D25" t="n">
-        <v>3.19</v>
+        <v>3.14</v>
       </c>
       <c r="E25" t="n">
-        <v>2.98</v>
+        <v>2.92</v>
       </c>
       <c r="F25" t="n">
-        <v>4.017</v>
+        <v>3.757</v>
       </c>
       <c r="G25" t="n">
-        <v>4.482</v>
+        <v>4.329</v>
       </c>
       <c r="H25" t="n">
-        <v>4.653</v>
+        <v>4.403</v>
       </c>
       <c r="I25" t="n">
-        <v>3.952</v>
+        <v>3.79</v>
       </c>
       <c r="J25" t="n">
-        <v>3.64</v>
+        <v>3.65</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C26" t="n">
         <v>2.92</v>
       </c>
       <c r="D26" t="n">
-        <v>3.19</v>
+        <v>3.14</v>
       </c>
       <c r="E26" t="n">
-        <v>2.98</v>
+        <v>2.92</v>
       </c>
       <c r="F26" t="n">
-        <v>3.996</v>
+        <v>3.736</v>
       </c>
       <c r="G26" t="n">
-        <v>4.414</v>
+        <v>4.29</v>
       </c>
       <c r="H26" t="n">
-        <v>4.57</v>
+        <v>4.361</v>
       </c>
       <c r="I26" t="n">
-        <v>3.867</v>
+        <v>3.74</v>
       </c>
       <c r="J26" t="n">
-        <v>3.64</v>
+        <v>3.65</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C27" t="n">
         <v>2.92</v>
       </c>
       <c r="D27" t="n">
-        <v>3.19</v>
+        <v>3.15</v>
       </c>
       <c r="E27" t="n">
-        <v>2.98</v>
+        <v>2.93</v>
       </c>
       <c r="F27" t="n">
-        <v>3.987</v>
+        <v>3.739</v>
       </c>
       <c r="G27" t="n">
-        <v>4.386</v>
+        <v>4.269</v>
       </c>
       <c r="H27" t="n">
-        <v>4.532</v>
+        <v>4.341</v>
       </c>
       <c r="I27" t="n">
-        <v>3.83</v>
+        <v>3.715</v>
       </c>
       <c r="J27" t="n">
-        <v>3.64</v>
+        <v>3.69</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C28" t="n">
         <v>2.92</v>
       </c>
       <c r="D28" t="n">
-        <v>3.19</v>
+        <v>3.16</v>
       </c>
       <c r="E28" t="n">
-        <v>2.98</v>
+        <v>2.94</v>
       </c>
       <c r="F28" t="n">
-        <v>3.981</v>
+        <v>3.751</v>
       </c>
       <c r="G28" t="n">
-        <v>4.371</v>
+        <v>4.259</v>
       </c>
       <c r="H28" t="n">
-        <v>4.505</v>
+        <v>4.333</v>
       </c>
       <c r="I28" t="n">
-        <v>3.803</v>
+        <v>3.7</v>
       </c>
       <c r="J28" t="n">
-        <v>3.65</v>
+        <v>3.63</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C29" t="n">
         <v>2.92</v>
       </c>
       <c r="D29" t="n">
-        <v>3.19</v>
+        <v>3.16</v>
       </c>
       <c r="E29" t="n">
-        <v>2.98</v>
+        <v>2.94</v>
       </c>
       <c r="F29" t="n">
-        <v>3.991</v>
+        <v>3.776</v>
       </c>
       <c r="G29" t="n">
+        <v>4.304</v>
+      </c>
+      <c r="H29" t="n">
         <v>4.386</v>
       </c>
-      <c r="H29" t="n">
-        <v>4.528</v>
-      </c>
       <c r="I29" t="n">
-        <v>3.827</v>
+        <v>3.752</v>
       </c>
       <c r="J29" t="n">
-        <v>3.65</v>
+        <v>3.63</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C30" t="n">
-        <v>2.95</v>
+        <v>2.92</v>
       </c>
       <c r="D30" t="n">
-        <v>3.19</v>
+        <v>3.16</v>
       </c>
       <c r="E30" t="n">
-        <v>2.98</v>
+        <v>2.94</v>
       </c>
       <c r="F30" t="n">
-        <v>3.974</v>
+        <v>3.817</v>
       </c>
       <c r="G30" t="n">
-        <v>4.347</v>
+        <v>4.337</v>
       </c>
       <c r="H30" t="n">
-        <v>4.461</v>
+        <v>4.418</v>
       </c>
       <c r="I30" t="n">
-        <v>3.76</v>
+        <v>3.782</v>
       </c>
       <c r="J30" t="n">
-        <v>3.65</v>
+        <v>3.62</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C31" t="n">
-        <v>2.95</v>
+        <v>2.92</v>
       </c>
       <c r="D31" t="n">
-        <v>3.19</v>
+        <v>3.16</v>
       </c>
       <c r="E31" t="n">
-        <v>2.98</v>
+        <v>2.94</v>
       </c>
       <c r="F31" t="n">
-        <v>3.974</v>
+        <v>3.817</v>
       </c>
       <c r="G31" t="n">
-        <v>4.347</v>
+        <v>4.337</v>
       </c>
       <c r="H31" t="n">
-        <v>4.461</v>
+        <v>4.418</v>
       </c>
       <c r="I31" t="n">
-        <v>3.76</v>
+        <v>3.782</v>
       </c>
       <c r="J31" t="n">
-        <v>3.65</v>
+        <v>3.62</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C32" t="n">
-        <v>2.95</v>
+        <v>2.92</v>
       </c>
       <c r="D32" t="n">
-        <v>3.19</v>
+        <v>3.16</v>
       </c>
       <c r="E32" t="n">
-        <v>2.98</v>
+        <v>2.94</v>
       </c>
       <c r="F32" t="n">
-        <v>3.974</v>
+        <v>3.817</v>
       </c>
       <c r="G32" t="n">
-        <v>4.347</v>
+        <v>4.337</v>
       </c>
       <c r="H32" t="n">
-        <v>4.461</v>
+        <v>4.418</v>
       </c>
       <c r="I32" t="n">
-        <v>3.76</v>
+        <v>3.782</v>
       </c>
       <c r="J32" t="n">
-        <v>3.65</v>
+        <v>3.62</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C33" t="n">
-        <v>2.93</v>
+        <v>2.92</v>
       </c>
       <c r="D33" t="n">
-        <v>3.19</v>
+        <v>3.16</v>
       </c>
       <c r="E33" t="n">
-        <v>2.98</v>
+        <v>2.95</v>
       </c>
       <c r="F33" t="n">
-        <v>3.964</v>
+        <v>3.843</v>
       </c>
       <c r="G33" t="n">
-        <v>4.331</v>
+        <v>4.364</v>
       </c>
       <c r="H33" t="n">
-        <v>4.443</v>
+        <v>4.446</v>
       </c>
       <c r="I33" t="n">
-        <v>3.742</v>
+        <v>3.805</v>
       </c>
       <c r="J33" t="n">
-        <v>3.66</v>
+        <v>3.62</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C34" t="n">
-        <v>2.93</v>
+        <v>2.92</v>
       </c>
       <c r="D34" t="n">
-        <v>3.19</v>
+        <v>3.17</v>
       </c>
       <c r="E34" t="n">
-        <v>2.98</v>
+        <v>2.95</v>
       </c>
       <c r="F34" t="n">
-        <v>3.962</v>
+        <v>3.841</v>
       </c>
       <c r="G34" t="n">
-        <v>4.343</v>
+        <v>4.35</v>
       </c>
       <c r="H34" t="n">
-        <v>4.441</v>
+        <v>4.411</v>
       </c>
       <c r="I34" t="n">
-        <v>3.74</v>
+        <v>3.765</v>
       </c>
       <c r="J34" t="n">
-        <v>3.65</v>
+        <v>3.61</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C35" t="n">
-        <v>2.93</v>
+        <v>2.92</v>
       </c>
       <c r="D35" t="n">
-        <v>3.19</v>
+        <v>3.18</v>
       </c>
       <c r="E35" t="n">
-        <v>2.98</v>
+        <v>2.96</v>
       </c>
       <c r="F35" t="n">
-        <v>3.943</v>
+        <v>3.869</v>
       </c>
       <c r="G35" t="n">
-        <v>4.273</v>
+        <v>4.366</v>
       </c>
       <c r="H35" t="n">
-        <v>4.38</v>
+        <v>4.427</v>
       </c>
       <c r="I35" t="n">
-        <v>3.677</v>
+        <v>3.775</v>
       </c>
       <c r="J35" t="n">
-        <v>3.66</v>
+        <v>3.62</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C36" t="n">
-        <v>2.93</v>
+        <v>2.92</v>
       </c>
       <c r="D36" t="n">
         <v>3.19</v>
       </c>
       <c r="E36" t="n">
-        <v>2.98</v>
+        <v>2.97</v>
       </c>
       <c r="F36" t="n">
-        <v>3.946</v>
+        <v>3.883</v>
       </c>
       <c r="G36" t="n">
-        <v>4.308</v>
+        <v>4.363</v>
       </c>
       <c r="H36" t="n">
-        <v>4.441</v>
+        <v>4.425</v>
       </c>
       <c r="I36" t="n">
-        <v>3.745</v>
+        <v>3.762</v>
       </c>
       <c r="J36" t="n">
-        <v>3.64</v>
+        <v>3.62</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C37" t="n">
-        <v>2.93</v>
+        <v>2.92</v>
       </c>
       <c r="D37" t="n">
-        <v>3.19</v>
+        <v>3.2</v>
       </c>
       <c r="E37" t="n">
-        <v>2.99</v>
+        <v>2.98</v>
       </c>
       <c r="F37" t="n">
-        <v>3.944</v>
+        <v>3.898</v>
       </c>
       <c r="G37" t="n">
-        <v>4.308</v>
+        <v>4.34</v>
       </c>
       <c r="H37" t="n">
-        <v>4.441</v>
+        <v>4.389</v>
       </c>
       <c r="I37" t="n">
-        <v>3.747</v>
+        <v>3.716</v>
       </c>
       <c r="J37" t="n">
-        <v>3.65</v>
+        <v>3.64</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C38" t="n">
-        <v>2.93</v>
+        <v>2.92</v>
       </c>
       <c r="D38" t="n">
-        <v>3.19</v>
+        <v>3.2</v>
       </c>
       <c r="E38" t="n">
-        <v>2.99</v>
+        <v>2.98</v>
       </c>
       <c r="F38" t="n">
-        <v>3.944</v>
+        <v>3.898</v>
       </c>
       <c r="G38" t="n">
-        <v>4.308</v>
+        <v>4.34</v>
       </c>
       <c r="H38" t="n">
-        <v>4.441</v>
+        <v>4.389</v>
       </c>
       <c r="I38" t="n">
-        <v>3.747</v>
+        <v>3.716</v>
       </c>
       <c r="J38" t="n">
-        <v>3.65</v>
+        <v>3.62</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C39" t="n">
-        <v>2.93</v>
+        <v>2.92</v>
       </c>
       <c r="D39" t="n">
-        <v>3.19</v>
+        <v>3.2</v>
       </c>
       <c r="E39" t="n">
-        <v>2.99</v>
+        <v>2.98</v>
       </c>
       <c r="F39" t="n">
-        <v>3.944</v>
+        <v>3.898</v>
       </c>
       <c r="G39" t="n">
-        <v>4.308</v>
+        <v>4.34</v>
       </c>
       <c r="H39" t="n">
-        <v>4.441</v>
+        <v>4.389</v>
       </c>
       <c r="I39" t="n">
-        <v>3.747</v>
+        <v>3.716</v>
       </c>
       <c r="J39" t="n">
-        <v>3.65</v>
+        <v>3.62</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C40" t="n">
-        <v>2.93</v>
+        <v>2.92</v>
       </c>
       <c r="D40" t="n">
-        <v>3.19</v>
+        <v>3.2</v>
       </c>
       <c r="E40" t="n">
         <v>2.99</v>
       </c>
       <c r="F40" t="n">
-        <v>3.958</v>
+        <v>3.927</v>
       </c>
       <c r="G40" t="n">
-        <v>4.324</v>
+        <v>4.36</v>
       </c>
       <c r="H40" t="n">
-        <v>4.465</v>
+        <v>4.412</v>
       </c>
       <c r="I40" t="n">
-        <v>3.775</v>
+        <v>3.735</v>
       </c>
       <c r="J40" t="n">
         <v>3.62</v>
@@ -1819,576 +1819,576 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C41" t="n">
-        <v>2.93</v>
+        <v>2.92</v>
       </c>
       <c r="D41" t="n">
-        <v>3.19</v>
+        <v>3.21</v>
       </c>
       <c r="E41" t="n">
         <v>2.99</v>
       </c>
       <c r="F41" t="n">
-        <v>3.971</v>
+        <v>3.951</v>
       </c>
       <c r="G41" t="n">
-        <v>4.357</v>
+        <v>4.344</v>
       </c>
       <c r="H41" t="n">
-        <v>4.486</v>
+        <v>4.38</v>
       </c>
       <c r="I41" t="n">
-        <v>3.797</v>
+        <v>3.697</v>
       </c>
       <c r="J41" t="n">
-        <v>3.63</v>
+        <v>3.62</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C42" t="n">
-        <v>2.93</v>
+        <v>2.92</v>
       </c>
       <c r="D42" t="n">
-        <v>3.19</v>
+        <v>3.21</v>
       </c>
       <c r="E42" t="n">
-        <v>2.99</v>
+        <v>2.98</v>
       </c>
       <c r="F42" t="n">
-        <v>3.962</v>
+        <v>3.987</v>
       </c>
       <c r="G42" t="n">
-        <v>4.341</v>
+        <v>4.432</v>
       </c>
       <c r="H42" t="n">
-        <v>4.471</v>
+        <v>4.472</v>
       </c>
       <c r="I42" t="n">
-        <v>3.782</v>
+        <v>3.791</v>
       </c>
       <c r="J42" t="n">
-        <v>3.64</v>
+        <v>3.68</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C43" t="n">
-        <v>2.93</v>
+        <v>2.92</v>
       </c>
       <c r="D43" t="n">
-        <v>3.19</v>
+        <v>3.2</v>
       </c>
       <c r="E43" t="n">
-        <v>2.99</v>
+        <v>2.97</v>
       </c>
       <c r="F43" t="n">
-        <v>3.961</v>
+        <v>3.974</v>
       </c>
       <c r="G43" t="n">
-        <v>4.348</v>
+        <v>4.401</v>
       </c>
       <c r="H43" t="n">
-        <v>4.464</v>
+        <v>4.434</v>
       </c>
       <c r="I43" t="n">
-        <v>3.777</v>
+        <v>3.745</v>
       </c>
       <c r="J43" t="n">
-        <v>3.62</v>
+        <v>3.66</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C44" t="n">
-        <v>2.93</v>
+        <v>2.92</v>
       </c>
       <c r="D44" t="n">
         <v>3.19</v>
       </c>
       <c r="E44" t="n">
-        <v>2.99</v>
+        <v>2.96</v>
       </c>
       <c r="F44" t="n">
-        <v>3.949</v>
+        <v>3.973</v>
       </c>
       <c r="G44" t="n">
-        <v>4.357</v>
+        <v>4.4</v>
       </c>
       <c r="H44" t="n">
-        <v>4.477</v>
+        <v>4.437</v>
       </c>
       <c r="I44" t="n">
-        <v>3.795</v>
+        <v>3.745</v>
       </c>
       <c r="J44" t="n">
-        <v>3.62</v>
+        <v>3.64</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C45" t="n">
-        <v>2.93</v>
+        <v>2.92</v>
       </c>
       <c r="D45" t="n">
         <v>3.19</v>
       </c>
       <c r="E45" t="n">
-        <v>2.99</v>
+        <v>2.96</v>
       </c>
       <c r="F45" t="n">
-        <v>3.949</v>
+        <v>3.973</v>
       </c>
       <c r="G45" t="n">
-        <v>4.357</v>
+        <v>4.4</v>
       </c>
       <c r="H45" t="n">
-        <v>4.477</v>
+        <v>4.437</v>
       </c>
       <c r="I45" t="n">
-        <v>3.795</v>
+        <v>3.745</v>
       </c>
       <c r="J45" t="n">
-        <v>3.62</v>
+        <v>3.64</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C46" t="n">
-        <v>2.93</v>
+        <v>2.92</v>
       </c>
       <c r="D46" t="n">
         <v>3.19</v>
       </c>
       <c r="E46" t="n">
-        <v>2.99</v>
+        <v>2.96</v>
       </c>
       <c r="F46" t="n">
-        <v>3.949</v>
+        <v>3.973</v>
       </c>
       <c r="G46" t="n">
-        <v>4.357</v>
+        <v>4.4</v>
       </c>
       <c r="H46" t="n">
-        <v>4.477</v>
+        <v>4.437</v>
       </c>
       <c r="I46" t="n">
-        <v>3.795</v>
+        <v>3.745</v>
       </c>
       <c r="J46" t="n">
-        <v>3.62</v>
+        <v>3.64</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C47" t="n">
-        <v>2.93</v>
+        <v>2.92</v>
       </c>
       <c r="D47" t="n">
         <v>3.19</v>
       </c>
       <c r="E47" t="n">
-        <v>2.99</v>
+        <v>2.95</v>
       </c>
       <c r="F47" t="n">
-        <v>3.949</v>
+        <v>3.976</v>
       </c>
       <c r="G47" t="n">
-        <v>4.357</v>
+        <v>4.401</v>
       </c>
       <c r="H47" t="n">
-        <v>4.477</v>
+        <v>4.461</v>
       </c>
       <c r="I47" t="n">
-        <v>3.795</v>
+        <v>3.77</v>
       </c>
       <c r="J47" t="n">
-        <v>3.62</v>
+        <v>3.64</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C48" t="n">
-        <v>2.93</v>
+        <v>2.91</v>
       </c>
       <c r="D48" t="n">
-        <v>3.19</v>
+        <v>3.18</v>
       </c>
       <c r="E48" t="n">
-        <v>2.99</v>
+        <v>2.94</v>
       </c>
       <c r="F48" t="n">
-        <v>3.968</v>
+        <v>3.977</v>
       </c>
       <c r="G48" t="n">
-        <v>4.397</v>
+        <v>4.399</v>
       </c>
       <c r="H48" t="n">
-        <v>4.522</v>
+        <v>4.469</v>
       </c>
       <c r="I48" t="n">
-        <v>3.84</v>
+        <v>3.777</v>
       </c>
       <c r="J48" t="n">
-        <v>3.66</v>
+        <v>3.63</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C49" t="n">
-        <v>2.93</v>
+        <v>2.91</v>
       </c>
       <c r="D49" t="n">
-        <v>3.19</v>
+        <v>3.18</v>
       </c>
       <c r="E49" t="n">
-        <v>2.99</v>
+        <v>2.94</v>
       </c>
       <c r="F49" t="n">
-        <v>3.969</v>
+        <v>3.986</v>
       </c>
       <c r="G49" t="n">
-        <v>4.355</v>
+        <v>4.395</v>
       </c>
       <c r="H49" t="n">
-        <v>4.471</v>
+        <v>4.472</v>
       </c>
       <c r="I49" t="n">
-        <v>3.787</v>
+        <v>3.776</v>
       </c>
       <c r="J49" t="n">
-        <v>3.65</v>
+        <v>3.62</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C50" t="n">
+        <v>2.91</v>
+      </c>
+      <c r="D50" t="n">
+        <v>3.18</v>
+      </c>
+      <c r="E50" t="n">
         <v>2.93</v>
       </c>
-      <c r="D50" t="n">
-        <v>3.19</v>
-      </c>
-      <c r="E50" t="n">
-        <v>2.99</v>
-      </c>
       <c r="F50" t="n">
-        <v>3.984</v>
+        <v>3.991</v>
       </c>
       <c r="G50" t="n">
-        <v>4.391</v>
+        <v>4.407</v>
       </c>
       <c r="H50" t="n">
-        <v>4.503</v>
+        <v>4.478</v>
       </c>
       <c r="I50" t="n">
-        <v>3.822</v>
+        <v>3.78</v>
       </c>
       <c r="J50" t="n">
-        <v>3.62</v>
+        <v>3.58</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C51" t="n">
-        <v>2.94</v>
+        <v>2.9</v>
       </c>
       <c r="D51" t="n">
-        <v>3.19</v>
+        <v>3.17</v>
       </c>
       <c r="E51" t="n">
-        <v>2.99</v>
+        <v>2.93</v>
       </c>
       <c r="F51" t="n">
-        <v>4.004</v>
+        <v>3.997</v>
       </c>
       <c r="G51" t="n">
-        <v>4.414</v>
+        <v>4.399</v>
       </c>
       <c r="H51" t="n">
-        <v>4.535</v>
+        <v>4.47</v>
       </c>
       <c r="I51" t="n">
-        <v>3.855</v>
+        <v>3.77</v>
       </c>
       <c r="J51" t="n">
-        <v>3.63</v>
+        <v>3.53</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C52" t="n">
-        <v>2.94</v>
+        <v>2.9</v>
       </c>
       <c r="D52" t="n">
-        <v>3.19</v>
+        <v>3.17</v>
       </c>
       <c r="E52" t="n">
-        <v>2.99</v>
+        <v>2.93</v>
       </c>
       <c r="F52" t="n">
-        <v>4.004</v>
+        <v>3.997</v>
       </c>
       <c r="G52" t="n">
-        <v>4.414</v>
+        <v>4.399</v>
       </c>
       <c r="H52" t="n">
-        <v>4.535</v>
+        <v>4.47</v>
       </c>
       <c r="I52" t="n">
-        <v>3.855</v>
+        <v>3.77</v>
       </c>
       <c r="J52" t="n">
-        <v>3.63</v>
+        <v>3.55</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C53" t="n">
-        <v>2.94</v>
+        <v>2.9</v>
       </c>
       <c r="D53" t="n">
-        <v>3.19</v>
+        <v>3.17</v>
       </c>
       <c r="E53" t="n">
-        <v>2.99</v>
+        <v>2.93</v>
       </c>
       <c r="F53" t="n">
-        <v>4.004</v>
+        <v>3.997</v>
       </c>
       <c r="G53" t="n">
-        <v>4.414</v>
+        <v>4.399</v>
       </c>
       <c r="H53" t="n">
-        <v>4.535</v>
+        <v>4.47</v>
       </c>
       <c r="I53" t="n">
-        <v>3.855</v>
+        <v>3.77</v>
       </c>
       <c r="J53" t="n">
-        <v>3.63</v>
+        <v>3.55</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C54" t="n">
-        <v>2.95</v>
+        <v>2.9</v>
       </c>
       <c r="D54" t="n">
-        <v>3.19</v>
+        <v>3.17</v>
       </c>
       <c r="E54" t="n">
-        <v>2.99</v>
+        <v>2.92</v>
       </c>
       <c r="F54" t="n">
-        <v>4.006</v>
+        <v>4.009</v>
       </c>
       <c r="G54" t="n">
-        <v>4.396</v>
+        <v>4.429</v>
       </c>
       <c r="H54" t="n">
-        <v>4.516</v>
+        <v>4.513</v>
       </c>
       <c r="I54" t="n">
-        <v>3.835</v>
+        <v>3.81</v>
       </c>
       <c r="J54" t="n">
-        <v>3.65</v>
+        <v>3.55</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C55" t="n">
-        <v>2.95</v>
+        <v>2.9</v>
       </c>
       <c r="D55" t="n">
-        <v>3.19</v>
+        <v>3.17</v>
       </c>
       <c r="E55" t="n">
-        <v>2.99</v>
+        <v>2.92</v>
       </c>
       <c r="F55" t="n">
-        <v>4.013</v>
+        <v>4.036</v>
       </c>
       <c r="G55" t="n">
-        <v>4.383</v>
+        <v>4.489</v>
       </c>
       <c r="H55" t="n">
-        <v>4.508</v>
+        <v>4.594</v>
       </c>
       <c r="I55" t="n">
-        <v>3.826</v>
+        <v>3.89</v>
       </c>
       <c r="J55" t="n">
-        <v>3.65</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="C56" t="n">
-        <v>2.96</v>
+        <v>2.9</v>
       </c>
       <c r="D56" t="n">
-        <v>3.2</v>
+        <v>3.17</v>
       </c>
       <c r="E56" t="n">
-        <v>3</v>
+        <v>2.92</v>
       </c>
       <c r="F56" t="n">
-        <v>4.019</v>
+        <v>4.018</v>
       </c>
       <c r="G56" t="n">
-        <v>4.384</v>
+        <v>4.462</v>
       </c>
       <c r="H56" t="n">
-        <v>4.498</v>
+        <v>4.572</v>
       </c>
       <c r="I56" t="n">
-        <v>3.817</v>
+        <v>3.867</v>
       </c>
       <c r="J56" t="n">
-        <v>3.66</v>
+        <v>3.63</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="C57" t="n">
-        <v>3.12</v>
+        <v>2.9</v>
       </c>
       <c r="D57" t="n">
-        <v>3.23</v>
+        <v>3.17</v>
       </c>
       <c r="E57" t="n">
-        <v>3.12</v>
+        <v>2.97</v>
       </c>
       <c r="F57" t="n">
-        <v>4.014</v>
+        <v>3.992</v>
       </c>
       <c r="G57" t="n">
-        <v>4.322</v>
+        <v>4.424</v>
       </c>
       <c r="H57" t="n">
-        <v>4.433</v>
+        <v>4.554</v>
       </c>
       <c r="I57" t="n">
-        <v>3.75</v>
+        <v>3.852</v>
       </c>
       <c r="J57" t="n">
         <v>3.64</v>
@@ -2397,476 +2397,1904 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="C58" t="n">
-        <v>3.12</v>
+        <v>2.9</v>
       </c>
       <c r="D58" t="n">
-        <v>3.23</v>
+        <v>3.17</v>
       </c>
       <c r="E58" t="n">
-        <v>3.13</v>
+        <v>2.97</v>
       </c>
       <c r="F58" t="n">
-        <v>4.019</v>
+        <v>3.992</v>
       </c>
       <c r="G58" t="n">
-        <v>4.368</v>
+        <v>4.424</v>
       </c>
       <c r="H58" t="n">
-        <v>4.476</v>
+        <v>4.554</v>
       </c>
       <c r="I58" t="n">
-        <v>3.795</v>
+        <v>3.852</v>
       </c>
       <c r="J58" t="n">
-        <v>3.64</v>
+        <v>3.62</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="C59" t="n">
-        <v>3.12</v>
+        <v>2.9</v>
       </c>
       <c r="D59" t="n">
-        <v>3.23</v>
+        <v>3.17</v>
       </c>
       <c r="E59" t="n">
-        <v>3.13</v>
+        <v>2.97</v>
       </c>
       <c r="F59" t="n">
-        <v>4.019</v>
+        <v>3.992</v>
       </c>
       <c r="G59" t="n">
-        <v>4.368</v>
+        <v>4.424</v>
       </c>
       <c r="H59" t="n">
-        <v>4.476</v>
+        <v>4.554</v>
       </c>
       <c r="I59" t="n">
-        <v>3.795</v>
+        <v>3.852</v>
       </c>
       <c r="J59" t="n">
-        <v>3.64</v>
+        <v>3.59</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="C60" t="n">
-        <v>3.12</v>
+        <v>2.9</v>
       </c>
       <c r="D60" t="n">
-        <v>3.23</v>
+        <v>3.17</v>
       </c>
       <c r="E60" t="n">
-        <v>3.13</v>
+        <v>2.97</v>
       </c>
       <c r="F60" t="n">
-        <v>4.019</v>
+        <v>3.992</v>
       </c>
       <c r="G60" t="n">
-        <v>4.368</v>
+        <v>4.424</v>
       </c>
       <c r="H60" t="n">
-        <v>4.476</v>
+        <v>4.554</v>
       </c>
       <c r="I60" t="n">
-        <v>3.795</v>
+        <v>3.852</v>
       </c>
       <c r="J60" t="n">
-        <v>3.64</v>
+        <v>3.59</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="C61" t="n">
-        <v>3.12</v>
+        <v>2.91</v>
       </c>
       <c r="D61" t="n">
-        <v>3.23</v>
+        <v>3.18</v>
       </c>
       <c r="E61" t="n">
-        <v>3.13</v>
+        <v>2.98</v>
       </c>
       <c r="F61" t="n">
-        <v>4.028</v>
+        <v>4.003</v>
       </c>
       <c r="G61" t="n">
-        <v>4.402</v>
+        <v>4.452</v>
       </c>
       <c r="H61" t="n">
-        <v>4.519</v>
+        <v>4.599</v>
       </c>
       <c r="I61" t="n">
-        <v>3.84</v>
+        <v>3.897</v>
       </c>
       <c r="J61" t="n">
-        <v>3.65</v>
+        <v>3.59</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="C62" t="n">
-        <v>3.12</v>
+        <v>2.91</v>
       </c>
       <c r="D62" t="n">
-        <v>3.23</v>
+        <v>3.19</v>
       </c>
       <c r="E62" t="n">
-        <v>3.14</v>
+        <v>2.98</v>
       </c>
       <c r="F62" t="n">
-        <v>4.041</v>
+        <v>3.988</v>
       </c>
       <c r="G62" t="n">
-        <v>4.433</v>
+        <v>4.398</v>
       </c>
       <c r="H62" t="n">
-        <v>4.557</v>
+        <v>4.57</v>
       </c>
       <c r="I62" t="n">
-        <v>3.878</v>
+        <v>3.866</v>
       </c>
       <c r="J62" t="n">
-        <v>3.68</v>
+        <v>3.57</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="C63" t="n">
-        <v>3.12</v>
+        <v>2.91</v>
       </c>
       <c r="D63" t="n">
-        <v>3.23</v>
+        <v>3.19</v>
       </c>
       <c r="E63" t="n">
-        <v>3.15</v>
+        <v>2.98</v>
       </c>
       <c r="F63" t="n">
-        <v>4.049</v>
+        <v>3.999</v>
       </c>
       <c r="G63" t="n">
-        <v>4.469</v>
+        <v>4.444</v>
       </c>
       <c r="H63" t="n">
-        <v>4.612</v>
+        <v>4.617</v>
       </c>
       <c r="I63" t="n">
-        <v>3.935</v>
+        <v>3.915</v>
       </c>
       <c r="J63" t="n">
-        <v>3.66</v>
+        <v>3.61</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="C64" t="n">
-        <v>3.12</v>
+        <v>2.91</v>
       </c>
       <c r="D64" t="n">
-        <v>3.24</v>
+        <v>3.19</v>
       </c>
       <c r="E64" t="n">
-        <v>3.16</v>
+        <v>2.98</v>
       </c>
       <c r="F64" t="n">
-        <v>4.046</v>
+        <v>4.007</v>
       </c>
       <c r="G64" t="n">
-        <v>4.417</v>
+        <v>4.454</v>
       </c>
       <c r="H64" t="n">
-        <v>4.558</v>
+        <v>4.617</v>
       </c>
       <c r="I64" t="n">
-        <v>3.882</v>
+        <v>3.917</v>
       </c>
       <c r="J64" t="n">
-        <v>3.65</v>
+        <v>3.62</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="C65" t="n">
-        <v>3.12</v>
+        <v>2.91</v>
       </c>
       <c r="D65" t="n">
-        <v>3.24</v>
+        <v>3.19</v>
       </c>
       <c r="E65" t="n">
-        <v>3.16</v>
+        <v>2.98</v>
       </c>
       <c r="F65" t="n">
-        <v>4.048</v>
+        <v>4.017</v>
       </c>
       <c r="G65" t="n">
-        <v>4.411</v>
+        <v>4.482</v>
       </c>
       <c r="H65" t="n">
-        <v>4.558</v>
+        <v>4.653</v>
       </c>
       <c r="I65" t="n">
-        <v>3.885</v>
+        <v>3.952</v>
       </c>
       <c r="J65" t="n">
-        <v>3.66</v>
+        <v>3.64</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="C66" t="n">
-        <v>3.12</v>
+        <v>2.91</v>
       </c>
       <c r="D66" t="n">
-        <v>3.24</v>
+        <v>3.19</v>
       </c>
       <c r="E66" t="n">
-        <v>3.16</v>
+        <v>2.98</v>
       </c>
       <c r="F66" t="n">
-        <v>4.048</v>
+        <v>4.017</v>
       </c>
       <c r="G66" t="n">
-        <v>4.411</v>
+        <v>4.482</v>
       </c>
       <c r="H66" t="n">
-        <v>4.558</v>
+        <v>4.653</v>
       </c>
       <c r="I66" t="n">
-        <v>3.885</v>
+        <v>3.952</v>
       </c>
       <c r="J66" t="n">
-        <v>3.66</v>
+        <v>3.64</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="C67" t="n">
-        <v>3.12</v>
+        <v>2.91</v>
       </c>
       <c r="D67" t="n">
-        <v>3.24</v>
+        <v>3.19</v>
       </c>
       <c r="E67" t="n">
-        <v>3.16</v>
+        <v>2.98</v>
       </c>
       <c r="F67" t="n">
-        <v>4.048</v>
+        <v>4.017</v>
       </c>
       <c r="G67" t="n">
-        <v>4.411</v>
+        <v>4.482</v>
       </c>
       <c r="H67" t="n">
-        <v>4.558</v>
+        <v>4.653</v>
       </c>
       <c r="I67" t="n">
-        <v>3.885</v>
+        <v>3.952</v>
       </c>
       <c r="J67" t="n">
-        <v>3.66</v>
+        <v>3.64</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="C68" t="n">
-        <v>3.12</v>
+        <v>2.92</v>
       </c>
       <c r="D68" t="n">
-        <v>3.24</v>
+        <v>3.19</v>
       </c>
       <c r="E68" t="n">
-        <v>3.16</v>
+        <v>2.98</v>
       </c>
       <c r="F68" t="n">
-        <v>4.054</v>
+        <v>3.996</v>
       </c>
       <c r="G68" t="n">
-        <v>4.43</v>
+        <v>4.414</v>
       </c>
       <c r="H68" t="n">
         <v>4.57</v>
       </c>
       <c r="I68" t="n">
-        <v>3.897</v>
+        <v>3.867</v>
       </c>
       <c r="J68" t="n">
-        <v>3.65</v>
+        <v>3.64</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="C69" t="n">
-        <v>3.12</v>
+        <v>2.92</v>
       </c>
       <c r="D69" t="n">
-        <v>3.25</v>
+        <v>3.19</v>
       </c>
       <c r="E69" t="n">
-        <v>3.17</v>
+        <v>2.98</v>
       </c>
       <c r="F69" t="n">
-        <v>4.069</v>
+        <v>3.987</v>
       </c>
       <c r="G69" t="n">
-        <v>4.438</v>
+        <v>4.386</v>
       </c>
       <c r="H69" t="n">
-        <v>4.568</v>
+        <v>4.532</v>
       </c>
       <c r="I69" t="n">
-        <v>3.897</v>
+        <v>3.83</v>
       </c>
       <c r="J69" t="n">
-        <v>3.65</v>
+        <v>3.64</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="C70" t="n">
-        <v>3.12</v>
+        <v>2.92</v>
       </c>
       <c r="D70" t="n">
-        <v>3.25</v>
+        <v>3.19</v>
       </c>
       <c r="E70" t="n">
-        <v>3.18</v>
+        <v>2.98</v>
       </c>
       <c r="F70" t="n">
-        <v>4.078</v>
+        <v>3.981</v>
       </c>
       <c r="G70" t="n">
-        <v>4.445</v>
+        <v>4.371</v>
       </c>
       <c r="H70" t="n">
-        <v>4.58</v>
+        <v>4.505</v>
       </c>
       <c r="I70" t="n">
-        <v>3.91</v>
+        <v>3.803</v>
       </c>
       <c r="J70" t="n">
-        <v>3.64</v>
+        <v>3.65</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C71" t="n">
+        <v>2.92</v>
+      </c>
+      <c r="D71" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E71" t="n">
+        <v>2.98</v>
+      </c>
+      <c r="F71" t="n">
+        <v>3.991</v>
+      </c>
+      <c r="G71" t="n">
+        <v>4.386</v>
+      </c>
+      <c r="H71" t="n">
+        <v>4.528</v>
+      </c>
+      <c r="I71" t="n">
+        <v>3.827</v>
+      </c>
+      <c r="J71" t="n">
+        <v>3.65</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C72" t="n">
+        <v>2.95</v>
+      </c>
+      <c r="D72" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E72" t="n">
+        <v>2.98</v>
+      </c>
+      <c r="F72" t="n">
+        <v>3.974</v>
+      </c>
+      <c r="G72" t="n">
+        <v>4.347</v>
+      </c>
+      <c r="H72" t="n">
+        <v>4.461</v>
+      </c>
+      <c r="I72" t="n">
+        <v>3.76</v>
+      </c>
+      <c r="J72" t="n">
+        <v>3.65</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C73" t="n">
+        <v>2.95</v>
+      </c>
+      <c r="D73" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E73" t="n">
+        <v>2.98</v>
+      </c>
+      <c r="F73" t="n">
+        <v>3.974</v>
+      </c>
+      <c r="G73" t="n">
+        <v>4.347</v>
+      </c>
+      <c r="H73" t="n">
+        <v>4.461</v>
+      </c>
+      <c r="I73" t="n">
+        <v>3.76</v>
+      </c>
+      <c r="J73" t="n">
+        <v>3.66</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C74" t="n">
+        <v>2.95</v>
+      </c>
+      <c r="D74" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E74" t="n">
+        <v>2.98</v>
+      </c>
+      <c r="F74" t="n">
+        <v>3.974</v>
+      </c>
+      <c r="G74" t="n">
+        <v>4.347</v>
+      </c>
+      <c r="H74" t="n">
+        <v>4.461</v>
+      </c>
+      <c r="I74" t="n">
+        <v>3.76</v>
+      </c>
+      <c r="J74" t="n">
+        <v>3.66</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C75" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D75" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E75" t="n">
+        <v>2.98</v>
+      </c>
+      <c r="F75" t="n">
+        <v>3.964</v>
+      </c>
+      <c r="G75" t="n">
+        <v>4.331</v>
+      </c>
+      <c r="H75" t="n">
+        <v>4.443</v>
+      </c>
+      <c r="I75" t="n">
+        <v>3.742</v>
+      </c>
+      <c r="J75" t="n">
+        <v>3.66</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C76" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D76" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E76" t="n">
+        <v>2.98</v>
+      </c>
+      <c r="F76" t="n">
+        <v>3.962</v>
+      </c>
+      <c r="G76" t="n">
+        <v>4.343</v>
+      </c>
+      <c r="H76" t="n">
+        <v>4.441</v>
+      </c>
+      <c r="I76" t="n">
+        <v>3.74</v>
+      </c>
+      <c r="J76" t="n">
+        <v>3.65</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C77" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D77" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E77" t="n">
+        <v>2.98</v>
+      </c>
+      <c r="F77" t="n">
+        <v>3.943</v>
+      </c>
+      <c r="G77" t="n">
+        <v>4.273</v>
+      </c>
+      <c r="H77" t="n">
+        <v>4.38</v>
+      </c>
+      <c r="I77" t="n">
+        <v>3.677</v>
+      </c>
+      <c r="J77" t="n">
+        <v>3.66</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C78" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D78" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E78" t="n">
+        <v>2.98</v>
+      </c>
+      <c r="F78" t="n">
+        <v>3.946</v>
+      </c>
+      <c r="G78" t="n">
+        <v>4.308</v>
+      </c>
+      <c r="H78" t="n">
+        <v>4.441</v>
+      </c>
+      <c r="I78" t="n">
+        <v>3.745</v>
+      </c>
+      <c r="J78" t="n">
+        <v>3.64</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C79" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D79" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E79" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="F79" t="n">
+        <v>3.944</v>
+      </c>
+      <c r="G79" t="n">
+        <v>4.308</v>
+      </c>
+      <c r="H79" t="n">
+        <v>4.441</v>
+      </c>
+      <c r="I79" t="n">
+        <v>3.747</v>
+      </c>
+      <c r="J79" t="n">
+        <v>3.65</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C80" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D80" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E80" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="F80" t="n">
+        <v>3.944</v>
+      </c>
+      <c r="G80" t="n">
+        <v>4.308</v>
+      </c>
+      <c r="H80" t="n">
+        <v>4.441</v>
+      </c>
+      <c r="I80" t="n">
+        <v>3.747</v>
+      </c>
+      <c r="J80" t="n">
+        <v>3.62</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C81" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D81" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E81" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="F81" t="n">
+        <v>3.944</v>
+      </c>
+      <c r="G81" t="n">
+        <v>4.308</v>
+      </c>
+      <c r="H81" t="n">
+        <v>4.441</v>
+      </c>
+      <c r="I81" t="n">
+        <v>3.747</v>
+      </c>
+      <c r="J81" t="n">
+        <v>3.62</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C82" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D82" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E82" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="F82" t="n">
+        <v>3.958</v>
+      </c>
+      <c r="G82" t="n">
+        <v>4.324</v>
+      </c>
+      <c r="H82" t="n">
+        <v>4.465</v>
+      </c>
+      <c r="I82" t="n">
+        <v>3.775</v>
+      </c>
+      <c r="J82" t="n">
+        <v>3.62</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C83" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D83" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E83" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="F83" t="n">
+        <v>3.971</v>
+      </c>
+      <c r="G83" t="n">
+        <v>4.357</v>
+      </c>
+      <c r="H83" t="n">
+        <v>4.486</v>
+      </c>
+      <c r="I83" t="n">
+        <v>3.797</v>
+      </c>
+      <c r="J83" t="n">
+        <v>3.63</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C84" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D84" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E84" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="F84" t="n">
+        <v>3.962</v>
+      </c>
+      <c r="G84" t="n">
+        <v>4.341</v>
+      </c>
+      <c r="H84" t="n">
+        <v>4.471</v>
+      </c>
+      <c r="I84" t="n">
+        <v>3.782</v>
+      </c>
+      <c r="J84" t="n">
+        <v>3.64</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C85" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D85" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E85" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="F85" t="n">
+        <v>3.961</v>
+      </c>
+      <c r="G85" t="n">
+        <v>4.348</v>
+      </c>
+      <c r="H85" t="n">
+        <v>4.464</v>
+      </c>
+      <c r="I85" t="n">
+        <v>3.777</v>
+      </c>
+      <c r="J85" t="n">
+        <v>3.62</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C86" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D86" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E86" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="F86" t="n">
+        <v>3.949</v>
+      </c>
+      <c r="G86" t="n">
+        <v>4.357</v>
+      </c>
+      <c r="H86" t="n">
+        <v>4.477</v>
+      </c>
+      <c r="I86" t="n">
+        <v>3.795</v>
+      </c>
+      <c r="J86" t="n">
+        <v>3.62</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C87" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D87" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E87" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="F87" t="n">
+        <v>3.949</v>
+      </c>
+      <c r="G87" t="n">
+        <v>4.357</v>
+      </c>
+      <c r="H87" t="n">
+        <v>4.477</v>
+      </c>
+      <c r="I87" t="n">
+        <v>3.795</v>
+      </c>
+      <c r="J87" t="n">
+        <v>3.62</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C88" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D88" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E88" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="F88" t="n">
+        <v>3.949</v>
+      </c>
+      <c r="G88" t="n">
+        <v>4.357</v>
+      </c>
+      <c r="H88" t="n">
+        <v>4.477</v>
+      </c>
+      <c r="I88" t="n">
+        <v>3.795</v>
+      </c>
+      <c r="J88" t="n">
+        <v>3.62</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C89" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D89" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E89" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="F89" t="n">
+        <v>3.949</v>
+      </c>
+      <c r="G89" t="n">
+        <v>4.357</v>
+      </c>
+      <c r="H89" t="n">
+        <v>4.477</v>
+      </c>
+      <c r="I89" t="n">
+        <v>3.795</v>
+      </c>
+      <c r="J89" t="n">
+        <v>3.62</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C90" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D90" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E90" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="F90" t="n">
+        <v>3.968</v>
+      </c>
+      <c r="G90" t="n">
+        <v>4.397</v>
+      </c>
+      <c r="H90" t="n">
+        <v>4.522</v>
+      </c>
+      <c r="I90" t="n">
+        <v>3.84</v>
+      </c>
+      <c r="J90" t="n">
+        <v>3.66</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C91" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D91" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E91" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="F91" t="n">
+        <v>3.969</v>
+      </c>
+      <c r="G91" t="n">
+        <v>4.355</v>
+      </c>
+      <c r="H91" t="n">
+        <v>4.471</v>
+      </c>
+      <c r="I91" t="n">
+        <v>3.787</v>
+      </c>
+      <c r="J91" t="n">
+        <v>3.65</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C92" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D92" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E92" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="F92" t="n">
+        <v>3.984</v>
+      </c>
+      <c r="G92" t="n">
+        <v>4.391</v>
+      </c>
+      <c r="H92" t="n">
+        <v>4.503</v>
+      </c>
+      <c r="I92" t="n">
+        <v>3.822</v>
+      </c>
+      <c r="J92" t="n">
+        <v>3.62</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C93" t="n">
+        <v>2.94</v>
+      </c>
+      <c r="D93" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E93" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="F93" t="n">
+        <v>4.004</v>
+      </c>
+      <c r="G93" t="n">
+        <v>4.414</v>
+      </c>
+      <c r="H93" t="n">
+        <v>4.535</v>
+      </c>
+      <c r="I93" t="n">
+        <v>3.855</v>
+      </c>
+      <c r="J93" t="n">
+        <v>3.63</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C94" t="n">
+        <v>2.94</v>
+      </c>
+      <c r="D94" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E94" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="F94" t="n">
+        <v>4.004</v>
+      </c>
+      <c r="G94" t="n">
+        <v>4.414</v>
+      </c>
+      <c r="H94" t="n">
+        <v>4.535</v>
+      </c>
+      <c r="I94" t="n">
+        <v>3.855</v>
+      </c>
+      <c r="J94" t="n">
+        <v>3.65</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C95" t="n">
+        <v>2.94</v>
+      </c>
+      <c r="D95" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E95" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="F95" t="n">
+        <v>4.004</v>
+      </c>
+      <c r="G95" t="n">
+        <v>4.414</v>
+      </c>
+      <c r="H95" t="n">
+        <v>4.535</v>
+      </c>
+      <c r="I95" t="n">
+        <v>3.855</v>
+      </c>
+      <c r="J95" t="n">
+        <v>3.65</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C96" t="n">
+        <v>2.95</v>
+      </c>
+      <c r="D96" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E96" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="F96" t="n">
+        <v>4.006</v>
+      </c>
+      <c r="G96" t="n">
+        <v>4.396</v>
+      </c>
+      <c r="H96" t="n">
+        <v>4.516</v>
+      </c>
+      <c r="I96" t="n">
+        <v>3.835</v>
+      </c>
+      <c r="J96" t="n">
+        <v>3.65</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C97" t="n">
+        <v>2.95</v>
+      </c>
+      <c r="D97" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="E97" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="F97" t="n">
+        <v>4.013</v>
+      </c>
+      <c r="G97" t="n">
+        <v>4.383</v>
+      </c>
+      <c r="H97" t="n">
+        <v>4.508</v>
+      </c>
+      <c r="I97" t="n">
+        <v>3.826</v>
+      </c>
+      <c r="J97" t="n">
+        <v>3.65</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C98" t="n">
+        <v>2.96</v>
+      </c>
+      <c r="D98" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="E98" t="n">
+        <v>3</v>
+      </c>
+      <c r="F98" t="n">
+        <v>4.019</v>
+      </c>
+      <c r="G98" t="n">
+        <v>4.384</v>
+      </c>
+      <c r="H98" t="n">
+        <v>4.498</v>
+      </c>
+      <c r="I98" t="n">
+        <v>3.817</v>
+      </c>
+      <c r="J98" t="n">
+        <v>3.66</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>3</v>
+      </c>
+      <c r="C99" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="D99" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="E99" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="F99" t="n">
+        <v>4.014</v>
+      </c>
+      <c r="G99" t="n">
+        <v>4.322</v>
+      </c>
+      <c r="H99" t="n">
+        <v>4.433</v>
+      </c>
+      <c r="I99" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="J99" t="n">
+        <v>3.64</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>3</v>
+      </c>
+      <c r="C100" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="D100" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="E100" t="n">
+        <v>3.13</v>
+      </c>
+      <c r="F100" t="n">
+        <v>4.019</v>
+      </c>
+      <c r="G100" t="n">
+        <v>4.368</v>
+      </c>
+      <c r="H100" t="n">
+        <v>4.476</v>
+      </c>
+      <c r="I100" t="n">
+        <v>3.795</v>
+      </c>
+      <c r="J100" t="n">
+        <v>3.64</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
+        <v>3</v>
+      </c>
+      <c r="C101" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="D101" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="E101" t="n">
+        <v>3.13</v>
+      </c>
+      <c r="F101" t="n">
+        <v>4.019</v>
+      </c>
+      <c r="G101" t="n">
+        <v>4.368</v>
+      </c>
+      <c r="H101" t="n">
+        <v>4.476</v>
+      </c>
+      <c r="I101" t="n">
+        <v>3.795</v>
+      </c>
+      <c r="J101" t="n">
+        <v>3.65</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>3</v>
+      </c>
+      <c r="C102" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="D102" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="E102" t="n">
+        <v>3.13</v>
+      </c>
+      <c r="F102" t="n">
+        <v>4.019</v>
+      </c>
+      <c r="G102" t="n">
+        <v>4.368</v>
+      </c>
+      <c r="H102" t="n">
+        <v>4.476</v>
+      </c>
+      <c r="I102" t="n">
+        <v>3.795</v>
+      </c>
+      <c r="J102" t="n">
+        <v>3.65</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>3</v>
+      </c>
+      <c r="C103" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="D103" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="E103" t="n">
+        <v>3.13</v>
+      </c>
+      <c r="F103" t="n">
+        <v>4.028</v>
+      </c>
+      <c r="G103" t="n">
+        <v>4.402</v>
+      </c>
+      <c r="H103" t="n">
+        <v>4.519</v>
+      </c>
+      <c r="I103" t="n">
+        <v>3.84</v>
+      </c>
+      <c r="J103" t="n">
+        <v>3.65</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B104" t="n">
+        <v>3</v>
+      </c>
+      <c r="C104" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="D104" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="E104" t="n">
+        <v>3.14</v>
+      </c>
+      <c r="F104" t="n">
+        <v>4.041</v>
+      </c>
+      <c r="G104" t="n">
+        <v>4.433</v>
+      </c>
+      <c r="H104" t="n">
+        <v>4.557</v>
+      </c>
+      <c r="I104" t="n">
+        <v>3.878</v>
+      </c>
+      <c r="J104" t="n">
+        <v>3.68</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B105" t="n">
+        <v>3</v>
+      </c>
+      <c r="C105" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="D105" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="E105" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="F105" t="n">
+        <v>4.049</v>
+      </c>
+      <c r="G105" t="n">
+        <v>4.469</v>
+      </c>
+      <c r="H105" t="n">
+        <v>4.612</v>
+      </c>
+      <c r="I105" t="n">
+        <v>3.935</v>
+      </c>
+      <c r="J105" t="n">
+        <v>3.66</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B106" t="n">
+        <v>3</v>
+      </c>
+      <c r="C106" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="D106" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="E106" t="n">
+        <v>3.16</v>
+      </c>
+      <c r="F106" t="n">
+        <v>4.046</v>
+      </c>
+      <c r="G106" t="n">
+        <v>4.417</v>
+      </c>
+      <c r="H106" t="n">
+        <v>4.558</v>
+      </c>
+      <c r="I106" t="n">
+        <v>3.882</v>
+      </c>
+      <c r="J106" t="n">
+        <v>3.65</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B107" t="n">
+        <v>3</v>
+      </c>
+      <c r="C107" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="D107" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="E107" t="n">
+        <v>3.16</v>
+      </c>
+      <c r="F107" t="n">
+        <v>4.048</v>
+      </c>
+      <c r="G107" t="n">
+        <v>4.411</v>
+      </c>
+      <c r="H107" t="n">
+        <v>4.558</v>
+      </c>
+      <c r="I107" t="n">
+        <v>3.885</v>
+      </c>
+      <c r="J107" t="n">
+        <v>3.66</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B108" t="n">
+        <v>3</v>
+      </c>
+      <c r="C108" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="D108" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="E108" t="n">
+        <v>3.16</v>
+      </c>
+      <c r="F108" t="n">
+        <v>4.048</v>
+      </c>
+      <c r="G108" t="n">
+        <v>4.411</v>
+      </c>
+      <c r="H108" t="n">
+        <v>4.558</v>
+      </c>
+      <c r="I108" t="n">
+        <v>3.885</v>
+      </c>
+      <c r="J108" t="n">
+        <v>3.65</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B109" t="n">
+        <v>3</v>
+      </c>
+      <c r="C109" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="D109" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="E109" t="n">
+        <v>3.16</v>
+      </c>
+      <c r="F109" t="n">
+        <v>4.048</v>
+      </c>
+      <c r="G109" t="n">
+        <v>4.411</v>
+      </c>
+      <c r="H109" t="n">
+        <v>4.558</v>
+      </c>
+      <c r="I109" t="n">
+        <v>3.885</v>
+      </c>
+      <c r="J109" t="n">
+        <v>3.65</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B110" t="n">
+        <v>3</v>
+      </c>
+      <c r="C110" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="D110" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="E110" t="n">
+        <v>3.16</v>
+      </c>
+      <c r="F110" t="n">
+        <v>4.054</v>
+      </c>
+      <c r="G110" t="n">
+        <v>4.43</v>
+      </c>
+      <c r="H110" t="n">
+        <v>4.57</v>
+      </c>
+      <c r="I110" t="n">
+        <v>3.897</v>
+      </c>
+      <c r="J110" t="n">
+        <v>3.65</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B111" t="n">
+        <v>3</v>
+      </c>
+      <c r="C111" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="D111" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="E111" t="n">
+        <v>3.17</v>
+      </c>
+      <c r="F111" t="n">
+        <v>4.069</v>
+      </c>
+      <c r="G111" t="n">
+        <v>4.438</v>
+      </c>
+      <c r="H111" t="n">
+        <v>4.568</v>
+      </c>
+      <c r="I111" t="n">
+        <v>3.897</v>
+      </c>
+      <c r="J111" t="n">
+        <v>3.65</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B112" t="n">
+        <v>3</v>
+      </c>
+      <c r="C112" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="D112" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="E112" t="n">
+        <v>3.18</v>
+      </c>
+      <c r="F112" t="n">
+        <v>4.078</v>
+      </c>
+      <c r="G112" t="n">
+        <v>4.445</v>
+      </c>
+      <c r="H112" t="n">
+        <v>4.58</v>
+      </c>
+      <c r="I112" t="n">
+        <v>3.91</v>
+      </c>
+      <c r="J112" t="n">
+        <v>3.64</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
           <t>2026-09-10</t>
         </is>
       </c>
-      <c r="B71" t="n">
+      <c r="B113" t="n">
         <v>3</v>
       </c>
-      <c r="C71" t="n">
+      <c r="C113" t="n">
         <v>3.12</v>
       </c>
-      <c r="D71" t="n">
+      <c r="D113" t="n">
         <v>3.26</v>
       </c>
-      <c r="E71" t="n">
+      <c r="E113" t="n">
         <v>3.18</v>
       </c>
-      <c r="F71" t="n">
+      <c r="F113" t="n">
         <v>4.091</v>
       </c>
-      <c r="G71" t="n">
+      <c r="G113" t="n">
         <v>4.464</v>
       </c>
-      <c r="H71" t="n">
+      <c r="H113" t="n">
         <v>4.595</v>
       </c>
-      <c r="I71" t="n">
+      <c r="I113" t="n">
         <v>3.927</v>
       </c>
-      <c r="J71" t="n">
+      <c r="J113" t="n">
         <v>3.64</v>
       </c>
     </row>

</xml_diff>